<commit_message>
Switch to six pillars and hook-and-beats scripts; add first weekly ideas doc
- Scripts cut to hook, beats, closing thought, tagline slot and per-platform
  captions per CLAUDE.md (full versions archived in the sheet's archive tab)
- Pillars: drop Pattern Breaks, add AI for Your Family and NotebookLM
- Checker updated for the new structure; bans "not broken" framing
- First weekly ideas doc (sourced ideas per pillar + 15 taglines)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqY8QbXMfegJWDBpeB6XE4
</commit_message>
<xml_diff>
--- a/deliverables/AI_Dad_Launch_Plan.xlsx
+++ b/deliverables/AI_Dad_Launch_Plan.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -482,118 +482,130 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WHAT CHANGED TONIGHT</t>
+          <t>WHAT CHANGED (OCT 14)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>(1) Story corrected everywhere: the account never names the habit. The story is now: the same destructive patterns, over and over → you finally told your wife something had to change → that was the turning point → ADHD diagnosis and AI, all inside about a month, about two months ago. (2) All three scripts rewritten for filming at your gym, with specific details. Each script has a 'Detail check' row so you only say what's true. (3) Pillar 3 is now 'Late-Diagnosis Log', and every pillar has 15 ready-to-film ideas. (4) Bios sharpened with the trend terms from this sheet. (5) New 'Filming Logistics' section: tripod verdict and the gym-music copyright risk. (6) Re-check log at the end of Assumptions.</t>
+          <t>CLAUDE.md is now the rulebook. (1) Scripts cut to hooks, beats, a closing thought and a tagline slot; the full word-for-word versions are archived in their own tab. (2) Six pillars: Pattern Breaks is out; AI for Your Family and NotebookLM are in. (3) First weekly ideas doc is live: https://docs.google.com/document/d/1Zt2vil6u8qryobcELQzVL_rTAWwFum0dVBF9VJu464M/edit (3 researched ideas per pillar + 15 taglines). (4) A new doc lands every Sunday at 5 AM ET.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>NAME DECISION</t>
+          <t>WHAT CHANGED (OCT 13)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Go with AI DAD HEALTHY DAD. 'AI Dad Happy Dad' contains the whole of HAPPY DAD, a brand owned by Happy Dad, LLC (the Nelk / Full Send hard seltzer). It has live filings in Class 33 (hard seltzer) and a registration covering Class 25 (clothing and hats), about 23 filings in all, and it keeps adding new HAPPY ___ marks. It markets to young men on TikTok and Instagram, the same apps you'll be on. Search 'happy dad' and you get their product, not you. For 'Healthy Dad' I found no live federal trademark, and the full phrase 'AI Dad Healthy Dad' has zero search results. The acronym still spells A-D-H-D. Re-checked after tonight's story change: the call rests on trademark and search crowding, and neither changed.</t>
+          <t>(1) Story corrected everywhere: the account never names the habit. The story is now: the same destructive patterns, over and over → you finally told your wife something had to change → that was the turning point → ADHD diagnosis and AI, all inside about a month, about two months ago. (2) All three scripts rewritten for filming at your gym, with specific details. Each script has a 'Detail check' row so you only say what's true. (3) Pillar 3 is now 'Late-Diagnosis Log', and every pillar has 15 ready-to-film ideas. (4) Bios sharpened with the trend terms from this sheet. (5) New 'Filming Logistics' section: tripod verdict and the gym-music copyright risk. (6) Re-check log at the end of Assumptions.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ACTION BEFORE WED</t>
+          <t>NAME DECISION</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Tonight: (1) Claim @aidadhealthydad on TikTok and Instagram. Also grab @aidadhappydad as a free defensive hold, but don't post on it. (2) Register aidadhealthydad.com at any registrar, about $10-20/yr. (3) Run the 5 USPTO queries in the 'Trademark Detail' section yourself; this sandbox's network blocked tmsearch.uspto.gov. (4) Connect TikTok and Instagram to your Metricool brand. It's linked, but no social accounts are connected yet. (5) Pack the filming kit and read each script's Detail check row (see Filming Logistics).</t>
+          <t>Go with AI DAD HEALTHY DAD. 'AI Dad Happy Dad' contains the whole of HAPPY DAD, a brand owned by Happy Dad, LLC (the Nelk / Full Send hard seltzer). It has live filings in Class 33 (hard seltzer) and a registration covering Class 25 (clothing and hats), about 23 filings in all, and it keeps adding new HAPPY ___ marks. It markets to young men on TikTok and Instagram, the same apps you'll be on. Search 'happy dad' and you get their product, not you. For 'Healthy Dad' I found no live federal trademark, and the full phrase 'AI Dad Healthy Dad' has zero search results. The acronym still spells A-D-H-D. Re-checked after tonight's story change: the call rests on trademark and search crowding, and neither changed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>FILMING AT THE GYM</t>
+          <t>ACTION BEFORE WED</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Talk where the music isn't. Gym speakers play licensed music, your mic will pick it up, and TikTok and Instagram scan audio automatically. A muted talking video is a dead video. So: record talking parts in your car in the gym lot or a music-free corner, and use the gym floor for silent B-roll. Turn on TikTok's 'Music copyright check' on the posting page. A $20-40 tripod with a Bluetooth remote is worth buying.</t>
+          <t>Tonight: (1) Claim @aidadhealthydad on TikTok and Instagram. Also grab @aidadhappydad as a free defensive hold, but don't post on it. (2) Register aidadhealthydad.com at any registrar, about $10-20/yr. (3) Run the 5 USPTO queries in the 'Trademark Detail' section yourself; this sandbox's network blocked tmsearch.uspto.gov. (4) Connect TikTok and Instagram to your Metricool brand. It's linked, but no social accounts are connected yet. (5) Pack the filming kit and read each script's Detail check row (see Filming Logistics).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>POSTING STACK (phone-only)</t>
+          <t>FILMING AT THE GYM</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Write/tighten scripts in the Claude app → film at your gym on a $20-40 tripod with a noise-cancelling clip mic (DJI Mic Mini class, ~$79 on sale) → edit + auto-captions in CapCut (TikTok master) → re-caption/finish the Instagram version in Edits (Instagram's free editor, no watermark) → schedule/auto-publish both through Metricool (already connected) → check TikTok Creative Center and your own For You page 10 min a day for trends. No AI faces, AI voices, or AI eye-contact fixes. Raw stays raw.</t>
+          <t>Talk where the music isn't. Gym speakers play licensed music, your mic will pick it up, and TikTok and Instagram scan audio automatically. A muted talking video is a dead video. So: record talking parts in your car in the gym lot or a music-free corner, and use the gym floor for silent B-roll. Turn on TikTok's 'Music copyright check' on the posting page. A $20-40 tripod with a Bluetooth remote is worth buying.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>SEQUENCE</t>
+          <t>POSTING STACK (phone-only)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>TikTok first, every time. Repurpose to Instagram Reels about 24 hours later with a clean export (no TikTok watermark) and fresh captions. TikTok's For You feed ranks on content signals, not follower count, so a zero-follower account can reach people on day one. Instagram rewards originality and 'sends' (shares by DM), so post a native, clean upload rather than a repost.</t>
+          <t>Write/tighten scripts in the Claude app → film at your gym on a $20-40 tripod with a noise-cancelling clip mic (DJI Mic Mini class, ~$79 on sale) → edit + auto-captions in CapCut (TikTok master) → re-caption/finish the Instagram version in Edits (Instagram's free editor, no watermark) → schedule/auto-publish both through Metricool (already connected) → check TikTok Creative Center and your own For You page 10 min a day for trends. No AI faces, AI voices, or AI eye-contact fixes. Raw stays raw.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>TIMING</t>
+          <t>SEQUENCE</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>First post (Wed): TikTok at 7:30 AM ET, which leaves 45 minutes after the gym to edit and proof captions. From Thursday: TikTok at 7:00 AM ET, Instagram Reels the next morning at 8:00 AM ET (in line with Hootsuite's morning window and Hopper's 7-8 AM Reels finding). Week 3: test one evening slot (6-8 PM, Metricool's TikTok study). After about 3 weeks of posts, switch to Metricool's personalized 'Best times' for your own audience.</t>
+          <t>TikTok first, every time. Repurpose to Instagram Reels about 24 hours later with a clean export (no TikTok watermark) and fresh captions. TikTok's For You feed ranks on content signals, not follower count, so a zero-follower account can reach people on day one. Instagram rewards originality and 'sends' (shares by DM), so post a native, clean upload rather than a repost.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>FIRST POST</t>
+          <t>TIMING</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Post Script B ('The Acronym') first: it has the strongest 1-second hook and explains the channel. Post Script C ('5:40 AM') second and Script A ('The Parking Lot') third. Film all three Wednesday morning, and pin all three on TikTok (it allows 3 pinned videos). Captions are burned into every video.</t>
+          <t>First post (Wed): TikTok at 7:30 AM ET, which leaves 45 minutes after the gym to edit and proof captions. From Thursday: TikTok at 7:00 AM ET, Instagram Reels the next morning at 8:00 AM ET (in line with Hootsuite's morning window and Hopper's 7-8 AM Reels finding). Week 3: test one evening slot (6-8 PM, Metricool's TikTok study). After about 3 weeks of posts, switch to Metricool's personalized 'Best times' for your own audience.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>CONTENT PILLARS</t>
+          <t>FIRST POST</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>1) 5AM Brain: early mornings at the gym as ADHD regulation, not hustle. 2) AI External Brain: real prompts, real screens. 3) Late-Diagnosis Log: two months in, what the diagnosis changed and didn't. 4) Pattern Breaks: the loop, the sentence to your wife, repair. 5) ADHD Dad in the Wild: dry humor with one fix. 15 ideas each = 75 videos, about 15 weeks at 5 a week. Each video gives viewers one thing worth saving.</t>
+          <t>Post Script B ('The Acronym') first: it has the strongest 1-second hook and explains the channel. Post Script C ('5:40 AM') second and Script A ('The Parking Lot') third. Film all three Wednesday morning, and pin all three on TikTok (it allows 3 pinned videos). Captions are burned into every video.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>CONTENT PILLARS</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>1) 5AM Brain. 2) AI External Brain (incl. prompting as a skill and the will-NOT list). 3) Late-Diagnosis Log. 4) AI for Your Family. 5) ADHD Dad in the Wild. 6) NotebookLM (personal use cases, not tutorials). 15 starter ideas each, plus 3 freshly researched ideas per pillar in every Sunday doc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>WHAT I COULDN'T VERIFY</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>The sandbox only allows web search, so I couldn't directly query USPTO, domain registries, or TikTok/Instagram profile pages. Trademark findings come from indexed USPTO-data mirrors (Justia, Trademarkia, uspto.report, TTABVUE). Handle and domain status is 'no existing use found', not 'confirmed available'. Instagram reach penalties for muted audio come from third-party guides; Meta hasn't confirmed them. None of this is legal advice. Before you file a federal application, get a 1-hour clearance review from a trademark attorney.</t>
         </is>
@@ -623,7 +635,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>What's moving now in dad, parenting and ADHD content, and how to use it without becoming a trend account.</t>
+          <t>Snapshot from Oct 13. Fresh, sourced trend research now arrives every Sunday in the weekly ideas doc: https://docs.google.com/document/d/1Zt2vil6u8qryobcELQzVL_rTAWwFum0dVBF9VJu464M/edit</t>
         </is>
       </c>
     </row>
@@ -908,42 +920,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="68" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="69" customWidth="1" min="6" max="6"/>
+    <col width="51" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>All three are written for the recommended name. If you keep 'Happy', swap 'Healthy' → 'Happy'; nothing else changes.</t>
+          <t>Per CLAUDE.md: the hook is word for word; the middle is beats only, and you tell the story live in your own words. The full word-for-word versions are archived, unchanged, in the 'Archive: full scripts (Oct 13)' tab.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Story rule: the habit is never named, hinted at, or counted in days. The story is the pattern, the sentence to your wife, and what came after.</t>
+          <t>Structure: hook (first 3-5 s) → beats → closing thought (last ~2 s, changes per video) → your fixed tagline (same every video; pick it from the weekly ideas doc).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Details: every script ends with a 'Detail check' row. TRUE lines come from what you told me (or your own setup). SWAP lines are specifics I wrote to make it sound like a real person: keep the ones that are true for you, and replace the rest with your version.</t>
+          <t>Story rule: the habit is never named or hinted at. Beats give the shape; the real details are yours.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Length: 60-75 seconds after jump cuts. Captions: word-by-word captions burned in on every line (CapCut auto-captions, proofread). Big on-screen TEXT sits above the captions.</t>
+          <t>Captions (re-checked Oct 14): TikTok short and hook-first with 3-5 hashtags; Instagram longer, keyword in the first sentence, up to 5 targeted hashtags.</t>
         </is>
       </c>
     </row>
@@ -957,7 +969,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Recommended order: B first (Wed), C second (Thu), A third (Fri). Film all three Wednesday morning. Pin all three.</t>
+          <t>Recommended order: B first, C second, A third. Pin all three.</t>
         </is>
       </c>
     </row>
@@ -969,7 +981,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Beat</t>
+          <t>Part</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -984,19 +996,19 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>You say (word for word)</t>
+          <t>Hook (word for word) / beats / closing</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Shot / delivery</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>B: The Acronym (POST FIRST)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1006,684 +1018,234 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>0-4s</t>
+          <t>0-5s</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>One sentence to my wife. It's why this account exists.</t>
+          <t>AI Dad Healthy Dad → A.D.H.D.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>One sentence to my wife. Two months ago. It's the reason this account exists.</t>
+          <t>AI Dad. Healthy Dad. ... Did you miss it? My doctor did.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Driver's seat, gym lot, engine off, still dark. Phone on the dash at eye level. First word on frame one: no 'hey guys', no smile yet.</t>
+          <t>Outside the gym doors or in a stairwell, no speakers in earshot. Point at the text as it appears. Beat of silence before 'Did you miss it?'</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>B: The Acronym (POST FIRST)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>The loop</t>
+          <t>BEATS</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>4-15s</t>
+          <t>5-55s</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Same pattern. Same apology. Same 'this time's different.'</t>
+          <t>ADHD dad · late-diagnosed · AI as my external brain</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>For years I ran the same destructive patterns. Same mistake, same apology, same speech about how this time was different. I could've given that speech in my sleep. Not a flex.</t>
+          <t>Beats only; say it your way: (1) who you are: a dad at the gym before the house wakes up. (2) The shape of the story: the same patterns over and over → the moment you told your wife something had to change → diagnosis and AI inside about a month. (3) One real thing AI changed for you, the one you can't stop telling people about. (4) What this account is: mornings, AI as an external brain, AI for your family.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Dry on 'Not a flex.' Glance away, then back to the lens.</t>
+          <t>Energy: 'I need to tell you about this.' No apologizing for the ADHD.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>B: The Acronym (POST FIRST)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>The sentence</t>
+          <t>CLOSING THOUGHT</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>15-26s</t>
+          <t>~2s</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>“Something has to change. And I think it's me.”</t>
+          <t>Just diagnosed? You're right on time.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Then one night I skipped the speech and said, 'Something has to change. And I think it's me.' That was the turning point. One sentence I'd dodged for years.</t>
+          <t>Just got the diagnosis? You're right on time.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Slow down. Hold one full second of silence after 'And I think it's me.'</t>
+          <t>Changes per video.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>B: The Acronym (POST FIRST)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>The month</t>
+          <t>TAGLINE</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>26-40s</t>
+          <t>end</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Inside a month: ADHD diagnosis + AI</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Inside a month, a doctor said 'ADHD.' About me. It explained a lot. Excused none of it. And I started using AI for the stuff my brain drops. Last night it checked whether this channel's name was trademarked.</t>
+          <t>[Your fixed tagline: pick one of the 15 in the weekly ideas doc]</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Jump cut between sentences and keep the cuts. Half-smile on 'trademarked.'</t>
+          <t>Same every video.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>B: The Acronym (POST FIRST)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>The channel</t>
+          <t>TikTok caption</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>40-50s</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>AI Dad. Healthy Dad. (Check the first letters.)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>So: AI Dad, Healthy Dad. Yes, the first letters spell exactly what you think. I'm two months into learning my own brain, and I'll show you what's helping, and what isn't.</t>
+          <t>Read the first letters. 🧠 #adhddad #adultadhd #latediagnosedadhd #dadsoftiktok</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Small smirk on 'exactly what you think.' Then straight down the lens.</t>
+          <t>Short; the video does the work.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>B: The Acronym (POST FIRST)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Soft CTA</t>
+          <t>Instagram caption</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>50-62s</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Been there? 🚗 below. Got a sentence you haven't said yet? DMs open.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>If you've been there, drop a 🚗 in the comments. If you've got your own version of that sentence, the one you haven't said yet, DM me. I'll read it right here tomorrow, before I go in.</t>
+          <t>ADHD dad, diagnosed as an adult, and I need to tell you what AI did for my brain. AI Dad Healthy Dad: read the first letters. #adhddad #adultadhd #latediagnosedadhd #aitools #dadlife</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Open the car door on the last word and cut as it opens. That's your ending.</t>
+          <t>Keyword in the first sentence; 5 hashtags.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>C: 5:40 AM</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Post copy</t>
+          <t>HOOK</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0-4s</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Cover text: 'The sentence that changed everything (ADHD dad)'</t>
+          <t>5:40 AM. The only hour my ADHD brain is quiet.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>CAPTION: Late-diagnosed ADHD dad. Two months ago I told my wife something had to change. Inside a month: the diagnosis, and AI. This account is what happens next. Lived experience, not medical advice. #adhddad #latediagnosedadhd #adultadhd #adhd #dadsoftiktok #fatherhood</t>
+          <t>5:40 a.m. The only hour my ADHD brain isn't running fourteen tabs.</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Pillar: Pattern Breaks</t>
+          <t>Say your real time. Quietest corner, back to a wall, no mirrors.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>A: The Parking Lot</t>
+          <t>C: 5:40 AM</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Detail check</t>
+          <t>BEATS</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4-55s</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>TRUE (from you): the repeating patterns; telling your wife something had to change; that being the turning point; the diagnosis and AI inside about a month, about two months ago; the gym before the house wakes up. TRUE (from last night): AI checked whether the channel name was trademarked. SWAP if it isn't yours: 'for years'; the speech-in-my-sleep line; the exact words of your sentence (use your own; the hook works with any one sentence); 'one night'. ASSUMES you drive to the gym; if not, film on a bench outside the entrance.</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Read before filming. Your cue card is the On-screen TEXT column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>HOOK</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>0-3s</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>AI Dad Healthy Dad → A.D.H.D.</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>AI Dad. Healthy Dad. Read the first letters.</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Outside the gym doors or in a stairwell, with no speakers in earshot. Point up at the text as it appears. Deadpan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>The payoff</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>3-8s</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>I didn't notice either. A doctor did.</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>... Yeah. I didn't notice either. A doctor did. About me. Two months ago.</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>One beat of silence before 'Yeah.' This line is what makes people stay.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Who</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>8-18s</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>ADHD dad · late-diagnosed · at the gym before the house wakes up</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>I'm a dad. It's not even six, I'm at the gym before my house wakes up, and I'm finally learning why my brain does what it does.</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Each fact pops on screen as you say it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>The story</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>18-30s</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Same patterns → told my wife → turning point → diagnosis + AI</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Short version: same destructive patterns, over and over. Different week, same ending. Then I told my wife something had to change. That was the turning point. Inside a month: the diagnosis, and AI.</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Steady pace. Don't rush 'told my wife.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>The turn</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>30-40s</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>AI didn't fix me. It built me a 296-row spreadsheet.</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>AI didn't fix me. I asked it to help launch this account, and it built me a 296-row spreadsheet. I have ADHD. I've read row one.</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Hold up your phone with the sheet open for 2 seconds, then back to camera. Dry: the laugh is theirs, not yours.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Three things (SAVEABLE)</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>40-58s</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>1. The gym before the house wakes up
-2. AI as my external brain (real prompts)
-3. Dad life with a brain that finally has a name</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>So I asked for the short version. One: the gym before my house wakes up, the only quiet hour I get. Two: AI as my external brain, real prompts, real screens. Three: dad life with a brain that finally has a name. Including the parts I'm still bad at.</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Fingers up for 1-2-3; each item stacks on screen so people screenshot it. One second of muted B-roll per item: the gym clock, your phone screen, your gym bag.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Soft CTA</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>58-67s</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Just diagnosed? Wondering? Say hi 👇</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Dads: just got the diagnosis? Or watching this going 'hang on...'? Say hi in the comments. You don't need it figured out. I clearly don't.</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Small smile on 'I clearly don't.' End on the last word.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Post copy</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Cover text: 'AI Dad Healthy Dad = ADHD'</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>CAPTION: ADHD dad here. Late-diagnosed two months ago. At the gym before the house wakes up, using AI as my external brain, figuring the rest out on camera. Lived experience, not medical advice. #adhddad #latediagnosedadhd #adultadhd #adhdtiktok #dadsoftiktok #5amclub #ai</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Pillar: Intro / all</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>B: The Acronym (POST FIRST)</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Detail check</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>TRUE (from you): the acronym; diagnosed about two months ago; patterns → told your wife → turning point → diagnosis and AI inside about a month; the gym before the house wakes up. TRUE (from tonight): AI built you this launch spreadsheet, which has 296 rows as of Oct 13 (if you add rows, update the number or say 'a giant spreadsheet'). SWAP if it isn't yours: 'It's not even six' (say your real time); 'the only quiet hour I get'; the B-roll items (use what's actually there).</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Read before filming. Your cue card is the On-screen TEXT column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>C: 5:40 AM</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>HOOK</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>0-4s</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>5:40 AM. The only hour my ADHD brain shuts up.</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>5:40 a.m. The only hour my ADHD brain isn't running fourteen tabs.</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Between sets; a little out of breath is fine. Quietest corner, back to a wall, no mirrors. If gym music is audible on playback, re-record your lines in the car and use these shots as muted B-roll.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>C: 5:40 AM</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Who</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>4-15s</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>ADHD dad · told my wife something had to change · diagnosis + AI inside a month</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Quick version: I'm a dad. Years of the same destructive patterns. Two months ago I told my wife something had to change. Inside a month: an ADHD diagnosis, and AI.</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Sit on the bench. Wipe your face mid-sentence: it reads as real, and it's a natural jump-cut point.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>C: 5:40 AM</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>The insight</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>15-27s</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>It's not about doing MORE. Nobody needs anything from me yet.</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>This hour isn't about getting more done. It's that nobody needs anything from me yet. No questions. No notifications. No 'Dad, where's my...' One bar, one decision. Closest my brain gets to quiet.</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>Cut to muted B-roll on 'One bar': hands on the barbell, the plates, the empty floor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>C: 5:40 AM</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>The reset</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>27-32s</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>My checklist resets at 3 AM. Yesterday doesn't get a vote.</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>My checklist resets itself at 3 a.m. Yesterday doesn't get a vote.</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Optional 2-second shot of the checklist on your phone screen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>C: 5:40 AM</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>The 3 calls (SAVEABLE)</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>32-52s</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Between sets, 3 calls:
 1. The ONE thing that has to happen today
@@ -1691,110 +1253,334 @@
 3. One thing with my kids. Phone in a drawer.</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Between sets I make three calls before the day makes them for me. One: the one thing that has to happen today. One, not five. Two: when the old pattern's most likely to show up, and what I'll do instead. Three: one thing with my kids, phone in a drawer. Then AI nags me till bedtime.</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>Count on your fingers. Each item stacks on screen: this is the part people save.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Beats only: (1) why this hour: nobody needs anything from you yet. (2) What the gym does for your head, in your words (don't claim mornings are scientifically better; the research doesn't say that). (3) Walk through your 3 calls between sets. (4) How AI holds those 3 calls for you all day.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>The on-screen list is the part people save.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>C: 5:40 AM</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Channel + soft CTA</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>52-63s</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>AI Dad. Healthy Dad. What time did you get up?</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>This is AI Dad, Healthy Dad. The initials are on purpose. Up this early too? Drop the time you got up. If not, DM me what your mornings look like now. Rough is fine.</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Stand up, last line to camera, walk back to the bar. Cut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>CLOSING THOUGHT</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>~2s</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Yesterday doesn't get a vote.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Yesterday doesn't get a vote.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Changes per video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>C: 5:40 AM</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Post copy</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>TAGLINE</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Cover text: 'The 3 calls I make at 5:40 AM (ADHD dad)'</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>CAPTION: ADHD dad morning routine, but not for productivity. It's for getting ahead of my brain before the day starts. The 3 calls are on screen; save it for tomorrow. Lived experience, not medical advice. #adhddad #adhd #morningroutine #5amclub #adultadhd #dadsoftiktok #gymtok</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>Pillar: 5AM Brain</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>[Your fixed tagline: pick one of the 15 in the weekly ideas doc]</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Same every video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>C: 5:40 AM</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Detail check</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>TikTok caption</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>TRUE (from you): morning person; gym in the morning; patterns → told your wife → diagnosis and AI inside about a month. CHECK (from your own Make account, seen while I checked its Google access): an automation named 'Checklist – Daily 3am Refresh'. Keep the 3 a.m. line only if that really resets your checklist; cut it if you'd rather not share it. SWAP if it isn't yours: '5:40' (your real time; change the hook text and cover too); 'Dad, where's my...' (use what your kids actually ask); 'years' of patterns.</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Read before filming. Your cue card is the On-screen TEXT column.</t>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>5:40 a.m. brain check. #adhddad #5amclub #adhd #gymtok</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Short; the video does the work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>C: 5:40 AM</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Instagram caption</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>ADHD morning routine from a dad who gets to the gym before his house wakes up. Not for productivity: for a quiet brain. The 3 calls I make between sets are on screen. #adhddad #morningroutine #5amclub #adultadhd #adhd</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Keyword in the first sentence; 5 hashtags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>A: The Parking Lot</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>HOOK</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0-4s</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>One sentence to my wife. It's why this account exists.</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>One sentence to my wife. Two months ago. It's the reason this account exists.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Driver's seat, gym lot, engine off. First word on frame one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>A: The Parking Lot</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>BEATS</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>4-55s</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Same patterns → one sentence → diagnosis + AI</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Beats only: (1) the loop, in your words: the same patterns, again and again (never the specific habit). (2) The night you told her: say the sentence you actually said. (3) What happened next, fast: the diagnosis and AI inside about a month. (4) What you're building here, and why you're fired up about it.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Slow down on the sentence. Let it sit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>A: The Parking Lot</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>CLOSING THOUGHT</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>~2s</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Your sentence is shorter than you think.</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Your sentence is shorter than you think.</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Changes per video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>A: The Parking Lot</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>TAGLINE</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>[Your fixed tagline: pick one of the 15 in the weekly ideas doc]</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Same every video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>A: The Parking Lot</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>TikTok caption</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>The sentence that started all this. #adhddad #latediagnosedadhd #adultadhd #dadsoftiktok</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Short; the video does the work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>A: The Parking Lot</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Instagram caption</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Late-diagnosed ADHD dad: two months ago I told my wife something had to change. Inside a month I had a diagnosis and AI in my corner, and I need to tell you about it. #adhddad #latediagnosedadhd #adultadhd #adhd #fatherhood</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Keyword in the first sentence; 5 hashtags.</t>
         </is>
       </c>
     </row>
@@ -2046,20 +1832,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="68" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="41" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Weekly rhythm: Mon AI External Brain · Tue Pattern Breaks · Wed 5AM Brain · Thu ADHD Dad in the Wild · Fri Late-Diagnosis Log · Sat reply-to-comment video + IG carousel · Sun batch-film. 5 pillars × 15 ideas = 75 videos, about 15 weeks at 5 a week. Every video carries one saveable thing (prompt, checklist, or script).</t>
+          <t>Weekly rhythm: Mon AI External Brain · Tue AI for Your Family · Wed 5AM Brain · Thu ADHD Dad in the Wild · Fri Late-Diagnosis Log · Sat NotebookLM + reply-to-comment video · Sun batch-film (the weekly ideas doc lands at 5 AM ET). 6 pillars × 15 starter ideas; fresh researched ideas arrive every Sunday. Ideas are story shapes: you supply the real story live.</t>
         </is>
       </c>
     </row>
@@ -2081,7 +1867,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Ready-to-film ideas (15)</t>
+          <t>Starter ideas (15, story shapes)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2098,7 +1884,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Early mornings at the gym, before the house wakes up, as ADHD regulation, not hustle: quiet before demand, and decisions made before the day makes them for you.</t>
+          <t>Early mornings at the gym, before the house wakes up, as ADHD regulation, not hustle-culture grind.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -2139,7 +1925,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Exactly how you use AI for the ADHD gaps: starting, remembering, planning, follow-through. Real screens and real prompts, failures included.</t>
+          <t>Real prompts and screens showing how AI fills ADHD gaps, including the 'will NOT use AI for' list and prompting as a skill, taught with humor. Most households don't pay for AI yet (about 3%, Bank of America data), so the gap is the urgency.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -2154,15 +1940,15 @@
 3) The school flyer trick: photo of the flyer, AI turns it into reminders. Save: the 3-step workflow.
 4) The worry sort: voice-memo everything on my mind, and AI sorts it into today / this week / not mine. Save: the sorting prompt.
 5) I asked AI if my channel name was trademarked: what it found, and what it said I still had to check myself. Save: the 'verify it yourself' list.
-6) AI built me a 296-row spreadsheet. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
+6) AI built me a 309-row spreadsheet. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
 7) The 'am I sliding?' check-in: one sentence to AI when the old pattern starts, and it asks me 3 questions back. Save: the 3 questions.
 8) 'Remind me later' → a real calendar event in 10 seconds, hands-free. Save: the dictation phrasing that works.
 9) What I will NOT use AI for: talking to my kids, apologizing to my wife, health decisions. Save: my human-only list.
 10) AI as a body double: 'check on me every 10 minutes while I do the dishes'. Save: the prompt.
 11) The email I've been avoiding: AI writes the first sentence, I write the rest. Save: the prompt.
-12) Planning a kid's birthday backward from the date. Save: the backward-plan prompt.
+12) Prompting is a skill: the same ask, a lazy prompt vs. a good one, side by side. Save: the 3-part prompt.
 13) My lifting log builds itself every Saturday: the one boring thing I automated first (check: from your Make automation name). Save: how to pick your first automation.
-14) Prompts that made it worse: the 40-item list, the generic pep talk. Save: how to ask for less.
+14) Prompts that made it worse, played for laughs: the 40-item list, the generic pep talk. Save: how to ask for less.
 15) Getting ready for a doctor's appointment: AI organizes my notes and questions; the doctor gives the answers. Save: the appointment-prep prompt.</t>
         </is>
       </c>
@@ -2175,12 +1961,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>3. Late-Diagnosis Log (new; replaces the old pillar 3)</t>
+          <t>3. Late-Diagnosis Log</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Two months in and counting: what the ADHD diagnosis changed, what it didn't, and what you're still figuring out. Honest updates from a late-diagnosed dad. Lived experience, not medical advice.</t>
+          <t>Ongoing, honest updates on what the diagnosis changed and what it didn't. No wins/progress-tracker angle.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2190,7 +1976,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1) The week after the diagnosis: relief, then a weird kind of grief, then 'now what?' Save: what actually helped that week.
+          <t>1) The week after the diagnosis: what it was actually like, in your words. Save: what actually helped that week.
 2) Explained, not excused: the rule I set the day I found out. Save: the rule, in one line.
 3) What I thought ADHD looked like vs what it looks like on me. Save: my 5 surprises (not a checklist for diagnosing anyone).
 4) The questions I took to my appointment. Save: the list (bring your own to a doctor).
@@ -2209,48 +1995,48 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Weekly on Fridays. Same opener every time: 'Late-diagnosed, week [X].' Car or quiet corner.</t>
+          <t>Car or quiet corner. Lived experience, not medical advice.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>4. Pattern Breaks</t>
+          <t>4. AI for Your Family</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>The loop, the sentence to your wife, and the repair. Practical and specific. The pattern itself is never named, and the tools work for any pattern.</t>
+          <t>A dad using AI to solve a family problem he can't fix through effort alone: 'I don't have to fix everything myself; I can hand someone the right tool.'</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Scripts, sentences and formulas</t>
+          <t>The tool, the prompt, or the house rule</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1) The sentence that changed everything, and how to say yours. Save: 3 ways to start the conversation.
-2) The 3 signs my loop is starting: going quiet, skipping the gym, 'I'll deal with it tomorrow'. Save: build your own early-warning list.
-3) Apologies with an action attached. Save: the formula (what I did / what it cost you / what I'm doing differently by [date]).
-4) Why 'this time's different' never worked: promises vs systems. Save: turn one promise into one system.
-5) The first 10 minutes when the old pattern shows up. Save: my 10-minute plan.
-6) Telling your partner: what I'd do differently. Save: the do/don't list.
-7) 'I'll remember': why my wife stopped accepting it, and what replaced it. Save: the shared-list setup.
-8) Shame is not a strategy: why beating myself up kept the loop running. Save: the shame → next step swap.
-9) Patterns live in calendars: how to map when and where yours shows up (I share the method, not my map). Save: the 7-day pattern map.
-10) The friend I told second: accountability without a speech. Save: what to ask a friend for.
-11) Repair with your kids: saying sorry so a kid actually gets it. Save: the kid-sized repair script.
-12) What week 3 of breaking a pattern actually felt like. Save: what to expect.
-13) Replace, don't just remove: what I put in the gap. Save: the replacement list.
-14) The setback video: when the old pattern wins a round, what I do next (film it only when it's real). Save: the setback plan.
-15) Two months in: what's actually different at home. Save: 3 signs of progress that aren't perfection.</t>
+          <t>1) The reading podcast (flagship): your wife, a teacher, built a NotebookLM podcast that got your son reading. Tell it your way, with her OK.
+2) The family problem you couldn't fix by trying harder, and the tool that did.
+3) Hints, not answers: AI at homework time without it doing the homework.
+4) The family calendar that finally works: how AI built it and who keeps it.
+5) Picky eaters vs. a week of dinners: AI makes the plan, you make the call.
+6) The school email pile → a 3-line Sunday brief.
+7) A bedtime story with your kid's name in it, made together.
+8) Our house rules for kids and AI: what it can and can't do.
+9) Your wife's teacher trick: how she uses AI in her classroom (with her OK).
+10) A hard topic, kid-sized: AI helps you find the words; you say them.
+11) Planning a kid's birthday backward from the date.
+12) I don't have to fix everything myself: the handoff mindset.
+13) Setting a grandparent up with one useful AI tool.
+14) The chore chart the kids actually follow.
+15) A day trip planned for a family with ADHD energy.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Talking head, slower pace, car or quiet corner. Strong 'send this to your partner' potential (Instagram sends).</t>
+          <t>Talking head + screen or result shots. Family members only with their OK.</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2048,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Dry-humor everyday moments: lost keys, school forms, fourteen tabs at bedtime. Each one ends with one actual fix.</t>
+          <t>Dry-humor everyday chaos, one concrete fix per video. The easiest on-ramp for new viewers.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2291,34 +2077,75 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>POV / skit-lite / voiceover over B-roll. The easiest on-ramp for new viewers.</t>
+          <t>POV / skit-lite / voiceover over B-roll.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>6. NotebookLM</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Not a feature tutorial. Each video is one powerful, personal use case, told for the feeling, not the buttons.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>The use case itself</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>1) A podcast about my own ADHD story that says my name.
+2) My motivational-speaker playlist + my goals → a morning pep episode made for me.
+3) Two AI hosts debate my brain: the Debate format on my own story.
+4) Before the appointment: my notes and questions read back in plain language (the doctor still gives the answers).
+5) My wedding vows and old letters → an anniversary episode.
+6) A week of gym voice memos → what I actually learned this week.
+7) A podcast for me, one year from now.
+8) My kids' school year → an audio yearbook.
+9) Grandma's recipes → an audio cookbook the kids can listen to.
+10) Spotify used it for Wrapped. I used it for my brain.
+11) Let it critique my content plan (the Critique format) and take the hit on camera.
+12) A Video Overview of my week.
+13) Hearing my own story told by two strangers' voices: what that felt like.
+14) The reading podcast, part two: what the kid thinks of it (with OK).
+15) The one episode I'd play for every newly diagnosed dad.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Play a few seconds of the generated audio, then your reaction. Check the audio's music-free before posting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>Recurring format: Comment Answers</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Reply to the best comment or DM question with a video, so the audience fills your calendar for you.</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>The answer itself</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Use TikTok's 'reply with video' on the top question each week. Turn DM themes into posts (anonymized).</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Saturdays. Keeps you from running dry by week 2.</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Saturdays, alongside NotebookLM.</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2679,12 +2506,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Guardrails followed: no emails sent, nothing pushed to GitHub, nothing deleted. Repo changes are committed locally only.</t>
+          <t>Guardrails followed: no emails sent and nothing deleted. On Oct 14 you asked me to push, so the branch claude/ai-dad-happy-dad-launch-r4xdw5 is on GitHub with all its commits.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Push when you're ready.</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2889,6 +2716,91 @@
       <c r="C34" s="3" t="inlineStr">
         <is>
           <t>No change needed: the name call rests on trademark and search crowding, which didn't change, and the names, prices and times now match everywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Oct 14: CLAUDE.md adopted. Scripts now carry only the hook (word for word), beats, a closing thought and a tagline slot. The full versions are archived unchanged in the 'Archive: full scripts (Oct 13)' tab.</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>The archive's SWAP lines are invented details; don't film them as written.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Six pillars per CLAUDE.md. Pattern Breaks was dropped; the origin story still lives in Script A's beats.</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Its old starter ideas are gone from the main tab (they're in this sheet's version history).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Weekly research uses web search and third-party roundups, because this sandbox can't open TikTok Creative Center or Instagram. Every claim names its source, and a pillar with no verified trend says so (this week: NotebookLM).</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Check the 7-day hashtags in Creative Center yourself before filming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>The weekly doc is a new Google Doc every Sunday at 5 AM ET in your Drive, titled 'AI Dad Weekly Ideas · Week of ...'. A scheduled task (4:52 AM ET Sundays, first run Oct 18) starts a fresh cloud session that does the research and writes the doc; it never edits this sheet.</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>ONE-TIME SETUP: the task was created without a Google Drive connection or the repo attached (this session couldn't pass them on). In claude.ai, open the scheduled task 'AI Dad weekly ideas doc (Sun 5 AM ET)' and add the Google Drive connector and this repo. Until then it saves the doc as an HTML file instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>The tagline is a placeholder until you pick one of the 15; then it's fixed on every video.</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2903,12 +2815,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4043,15 +3955,236 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>CDC MMWR 73(40): ADHD in adults</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/73/wr/mm7340a1.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>ADDitude: half diagnosed in adulthood</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>https://www.additudemag.com/adult-adhd-diagnosis-cdc-report/</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>NPR: a handful of Americans pay for AI</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.npr.org/2026/06/04/nx-s1-5791661/chatgpt-gemini-claude-subscription-revenue-openai</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Moneywise: BofA, 3% of households pay for AI</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>https://moneywise.com/news/top-stories/ai-subscribers-households-bank-america-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>National Literacy Trust: AI and literacy 2026</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>https://literacytrust.org.uk/research-services/research-reports/young-people-teachers-and-parents-use-of-ai-to-support-literacy-in-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Digital Trends: parents worry about AI reliance</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>https://www.digitaltrends.com/computing/parents-fear-kids-are-becoming-too-dependent-on-ai-while-schools-struggle-to-keep-up-survey-finds/</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>JOGH 2025: physical activity and adult ADHD</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>https://jogh.org/2025/jogh-15-04025</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Single exercise session meta-analysis (2025)</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12220223/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>NotebookLM guide 2026 (Audio Overview formats)</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>https://toolchase.com/blog/notebooklm-complete-guide/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>NotebookLM (Wikipedia)</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/NotebookLM</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Instagram hashtags 2026 (Inro)</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.inro.social/blog/instagram-hashtags-relevant-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Caption length guide (SocialPilot)</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>https://www.socialpilot.co/blog/ideal-social-media-caption-length</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Oct 14)</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>TikTok trends October 2026 (Ramdam)</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ramd.am/blog/trends-tiktok</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
           <t>Filming</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>PureGym filming rule (STV News)</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="C82" s="3" t="inlineStr">
         <is>
           <t>https://news.stv.tv/world/gym-fluencers-urged-to-stop-filming-in-public-amid-privacy-concerns</t>
         </is>
@@ -6301,7 +6434,7 @@
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="43" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="57" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -6527,7 +6660,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Pattern Breaks</t>
+          <t>Late-Diagnosis Log</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -6623,7 +6756,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Pattern Breaks</t>
+          <t>Late-Diagnosis Log</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -6672,27 +6805,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
+          <t>5:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Weekly ideas doc lands; batch-film 3-4 videos</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Batch-film 3-4 videos for next week (pick from the 15-idea lists in Content Pillars)</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Morning gym session, 45 min</t>
+          <t>Pick from the doc and the starter lists</t>
         </is>
       </c>
     </row>
@@ -6746,17 +6879,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Pattern Breaks: 'Apologies with an action attached'</t>
+          <t>AI for Your Family: 'The reading podcast'</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Pattern Breaks</t>
+          <t>AI for Your Family</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Put the formula on screen; it's the saveable part</t>
+          <t>Flagship story. Hook from the weekly doc; you tell it live, with your wife's OK.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restructure the launch-plan sheet into a skimmable one-fact-per-row layout
The sheet layout now splits every long cell into short lines (by line
break, numbered item, arrow chain, sentence, then clause), one fact per
row, with each column reading straight down and a blank row between
records. Text is split, never reworded: a check confirms every cell's
words survive unchanged. Bio copy stays whole so it pastes exactly.

Also: two lines reworded so they don't start with a quote mark, the
row-count idea phrased to read right at any count, and assumption 35
updated now that the weekly routine is set up by hand.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqY8QbXMfegJWDBpeB6XE4
</commit_message>
<xml_diff>
--- a/deliverables/AI_Dad_Launch_Plan.xlsx
+++ b/deliverables/AI_Dad_Launch_Plan.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Go with AI DAD HEALTHY DAD. 'AI Dad Happy Dad' contains the whole of HAPPY DAD, a brand owned by Happy Dad, LLC (the Nelk / Full Send hard seltzer). It has live filings in Class 33 (hard seltzer) and a registration covering Class 25 (clothing and hats), about 23 filings in all, and it keeps adding new HAPPY ___ marks. It markets to young men on TikTok and Instagram, the same apps you'll be on. Search 'happy dad' and you get their product, not you. For 'Healthy Dad' I found no live federal trademark, and the full phrase 'AI Dad Healthy Dad' has zero search results. The acronym still spells A-D-H-D. Re-checked after tonight's story change: the call rests on trademark and search crowding, and neither changed.</t>
+          <t>Go with AI DAD HEALTHY DAD. The name 'AI Dad Happy Dad' contains the whole of HAPPY DAD, a brand owned by Happy Dad, LLC (the Nelk / Full Send hard seltzer). It has live filings in Class 33 (hard seltzer) and a registration covering Class 25 (clothing and hats), about 23 filings in all, and it keeps adding new HAPPY ___ marks. It markets to young men on TikTok and Instagram, the same apps you'll be on. Search 'happy dad' and you get their product, not you. For 'Healthy Dad' I found no live federal trademark, and the full phrase 'AI Dad Healthy Dad' has zero search results. The acronym still spells A-D-H-D. Re-checked after tonight's story change: the call rests on trademark and search crowding, and neither changed.</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
 3) The school flyer trick: photo of the flyer, AI turns it into reminders. Save: the 3-step workflow.
 4) The worry sort: voice-memo everything on my mind, and AI sorts it into today / this week / not mine. Save: the sorting prompt.
 5) I asked AI if my channel name was trademarked: what it found, and what it said I still had to check myself. Save: the 'verify it yourself' list.
-6) AI built me a 309-row spreadsheet. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
+6) AI built me a spreadsheet with 864 rows. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
 7) The 'am I sliding?' check-in: one sentence to AI when the old pattern starts, and it asks me 3 questions back. Save: the 3 questions.
 8) 'Remind me later' → a real calendar event in 10 seconds, hands-free. Save: the dictation phrasing that works.
 9) What I will NOT use AI for: talking to my kids, apologizing to my wife, health decisions. Save: my human-only list.
@@ -2778,12 +2778,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>The weekly doc is a new Google Doc every Sunday at 5 AM ET in your Drive, titled 'AI Dad Weekly Ideas · Week of ...'. A scheduled task (4:52 AM ET Sundays, first run Oct 18) starts a fresh cloud session that does the research and writes the doc; it never edits this sheet.</t>
+          <t>The weekly doc is a new Google Doc every Sunday at 5 AM ET in your Drive, titled 'AI Dad Weekly Ideas · Week of ...'. It comes from a routine you set up yourself at claude.ai/code/routines (Sundays 4:52 AM ET), using the prompt in docs/weekly_routine_prompt.md. It never edits this sheet.</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>ONE-TIME SETUP: the task was created without a Google Drive connection or the repo attached (this session couldn't pass them on). In claude.ai, open the scheduled task 'AI Dad weekly ideas doc (Sun 5 AM ET)' and add the Google Drive connector and this repo. Until then it saves the doc as an HTML file instead.</t>
+          <t>The scheduled task I first created didn't show up in your account, so I deleted it. Give the routine Google Drive as its only connector and attach this repo.</t>
         </is>
       </c>
     </row>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>No drinks-brand association. 'Healthy' fits a story about breaking patterns, early mornings and the gym.</t>
+          <t>No drinks-brand association. The word 'Healthy' fits a story about breaking patterns, early mornings and the gym.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Tease-then-reveal launch and one-doc-per-week guard for the weekly routine
- New Launch Phases section: 2-week, 12-post teaser phase (Oct 21 - Nov 3),
  reveal week Nov 4-7 with Scripts B, A, C, pillar rhythm from Nov 9, plus
  a reveal-early rule. Length is reasoned from new-account research,
  sources listed.
- Launch Calendar replaces Week 1 Calendar; teaser-phase bios added; the
  checker blocks mechanism words in teaser bios and story shapes.
- CLAUDE.md: Launch Phases rules, and a one-doc-per-week rule the weekly
  run applies before any research (REDO to regenerate; old doc renamed,
  never deleted).
- docs/weekly_routine_prompt.md: same guard as step 0, teaser handling,
  and a check-before-retry on doc creation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqY8QbXMfegJWDBpeB6XE4
</commit_message>
<xml_diff>
--- a/deliverables/AI_Dad_Launch_Plan.xlsx
+++ b/deliverables/AI_Dad_Launch_Plan.xlsx
@@ -15,13 +15,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Stack" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filming Logistics" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timing &amp; Sequence" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Calendar" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trends (Oct 2026)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripts" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bio" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pillars" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Phases" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Calendar" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trends (Oct 2026)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bio" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pillars" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -456,7 +457,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Dad ___ Dad: launch plan. Research done 2026-10-13; updated the night of Oct 13. First post: Wednesday, Oct 14, 2026, morning.</t>
+          <t>AI Dad ___ Dad: launch plan. Research done 2026-10-13; updated Oct 19: tease first, reveal on Wed Nov 4. First teaser post: Wednesday, Oct 21, 2026, morning.</t>
         </is>
       </c>
     </row>
@@ -482,130 +483,154 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WHAT CHANGED (OCT 14)</t>
+          <t>WHAT CHANGED (OCT 19)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>CLAUDE.md is now the rulebook. (1) Scripts cut to hooks, beats, a closing thought and a tagline slot; the full word-for-word versions are archived in their own tab. (2) Six pillars: Pattern Breaks is out; AI for Your Family and NotebookLM are in. (3) First weekly ideas doc is live: https://docs.google.com/document/d/1Zt2vil6u8qryobcELQzVL_rTAWwFum0dVBF9VJu464M/edit (3 researched ideas per pillar + 15 taglines). (4) A new doc lands every Sunday at 5 AM ET.</t>
+          <t>(1) Launch is now tease-then-reveal. For the first 2 weeks (12 posts, Wed Oct 21 to Tue Nov 3) you show real moments and results and never explain the why: no 'ADHD', no 'AI'. Wed Nov 4 is the reveal (Script B, 'The Acronym'). See the new 'Launch Phases' section for why 2 weeks. (2) The calendar is now the 'Launch Calendar'. (3) New teaser-phase bios. (4) The weekly routine can no longer create a second doc for the same week.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>WHAT CHANGED (OCT 13)</t>
+          <t>LAUNCH: TEASE FIRST</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>(1) Story corrected everywhere: the account never names the habit. The story is now: the same destructive patterns, over and over → you finally told your wife something had to change → that was the turning point → ADHD diagnosis and AI, all inside about a month, about two months ago. (2) All three scripts rewritten for filming at your gym, with specific details. Each script has a 'Detail check' row so you only say what's true. (3) Pillar 3 is now 'Late-Diagnosis Log', and every pillar has 15 ready-to-film ideas. (4) Bios sharpened with the trend terms from this sheet. (5) New 'Filming Logistics' section: tripod verdict and the gym-music copyright risk. (6) Re-check log at the end of Assumptions.</t>
+          <t>Weeks 1-2: results without the how. Week 3: the reveal. Each teaser must work on its own (a real moment, a real result, a clean ending) because a brand-new account's viewers mostly see one video, not the series. If people keep asking 'how?' in the comments, reveal early (rule in Launch Phases).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>NAME DECISION</t>
+          <t>WHAT CHANGED (OCT 14)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Go with AI DAD HEALTHY DAD. The name 'AI Dad Happy Dad' contains the whole of HAPPY DAD, a brand owned by Happy Dad, LLC (the Nelk / Full Send hard seltzer). It has live filings in Class 33 (hard seltzer) and a registration covering Class 25 (clothing and hats), about 23 filings in all, and it keeps adding new HAPPY ___ marks. It markets to young men on TikTok and Instagram, the same apps you'll be on. Search 'happy dad' and you get their product, not you. For 'Healthy Dad' I found no live federal trademark, and the full phrase 'AI Dad Healthy Dad' has zero search results. The acronym still spells A-D-H-D. Re-checked after tonight's story change: the call rests on trademark and search crowding, and neither changed.</t>
+          <t>CLAUDE.md is now the rulebook. (1) Scripts cut to hooks, beats, a closing thought and a tagline slot; the full word-for-word versions are archived in their own tab. (2) Six pillars: Pattern Breaks is out; AI for Your Family and NotebookLM are in. (3) First weekly ideas doc is live: https://docs.google.com/document/d/1Zt2vil6u8qryobcELQzVL_rTAWwFum0dVBF9VJu464M/edit (3 researched ideas per pillar + 15 taglines). (4) A new doc lands every Sunday at 5 AM ET.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>ACTION BEFORE WED</t>
+          <t>WHAT CHANGED (OCT 13)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Tonight: (1) Claim @aidadhealthydad on TikTok and Instagram. Also grab @aidadhappydad as a free defensive hold, but don't post on it. (2) Register aidadhealthydad.com at any registrar, about $10-20/yr. (3) Run the 5 USPTO queries in the 'Trademark Detail' section yourself; this sandbox's network blocked tmsearch.uspto.gov. (4) Connect TikTok and Instagram to your Metricool brand. It's linked, but no social accounts are connected yet. (5) Pack the filming kit and read each script's Detail check row (see Filming Logistics).</t>
+          <t>(1) Story corrected everywhere: the account never names the habit. The story is now: the same destructive patterns, over and over → you finally told your wife something had to change → that was the turning point → ADHD diagnosis and AI, all inside about a month, about two months ago. (2) All three scripts rewritten for filming at your gym, with specific details. Each script has a 'Detail check' row so you only say what's true. (3) Pillar 3 is now 'Late-Diagnosis Log', and every pillar has 15 ready-to-film ideas. (4) Bios sharpened with the trend terms from this sheet. (5) New 'Filming Logistics' section: tripod verdict and the gym-music copyright risk. (6) Re-check log at the end of Assumptions.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>FILMING AT THE GYM</t>
+          <t>NAME DECISION</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Talk where the music isn't. Gym speakers play licensed music, your mic will pick it up, and TikTok and Instagram scan audio automatically. A muted talking video is a dead video. So: record talking parts in your car in the gym lot or a music-free corner, and use the gym floor for silent B-roll. Turn on TikTok's 'Music copyright check' on the posting page. A $20-40 tripod with a Bluetooth remote is worth buying.</t>
+          <t>Go with AI DAD HEALTHY DAD. The name 'AI Dad Happy Dad' contains the whole of HAPPY DAD, a brand owned by Happy Dad, LLC (the Nelk / Full Send hard seltzer). It has live filings in Class 33 (hard seltzer) and a registration covering Class 25 (clothing and hats), about 23 filings in all, and it keeps adding new HAPPY ___ marks. It markets to young men on TikTok and Instagram, the same apps you'll be on. Search 'happy dad' and you get their product, not you. For 'Healthy Dad' I found no live federal trademark, and the full phrase 'AI Dad Healthy Dad' has zero search results. The acronym still spells A-D-H-D. Re-checked after tonight's story change: the call rests on trademark and search crowding, and neither changed.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>POSTING STACK (phone-only)</t>
+          <t>ACTION BEFORE WED</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Write/tighten scripts in the Claude app → film at your gym on a $20-40 tripod with a noise-cancelling clip mic (DJI Mic Mini class, ~$79 on sale) → edit + auto-captions in CapCut (TikTok master) → re-caption/finish the Instagram version in Edits (Instagram's free editor, no watermark) → schedule/auto-publish both through Metricool (already connected) → check TikTok Creative Center and your own For You page 10 min a day for trends. No AI faces, AI voices, or AI eye-contact fixes. Raw stays raw.</t>
+          <t>Tonight: (1) Claim @aidadhealthydad on TikTok and Instagram. Also grab @aidadhappydad as a free defensive hold, but don't post on it. (2) Register aidadhealthydad.com at any registrar, about $10-20/yr. (3) Run the 5 USPTO queries in the 'Trademark Detail' section yourself; this sandbox's network blocked tmsearch.uspto.gov. (4) Connect TikTok and Instagram to your Metricool brand. It's linked, but no social accounts are connected yet. (5) Pack the filming kit and read each script's Detail check row (see Filming Logistics).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>SEQUENCE</t>
+          <t>FILMING AT THE GYM</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>TikTok first, every time. Repurpose to Instagram Reels about 24 hours later with a clean export (no TikTok watermark) and fresh captions. TikTok's For You feed ranks on content signals, not follower count, so a zero-follower account can reach people on day one. Instagram rewards originality and 'sends' (shares by DM), so post a native, clean upload rather than a repost.</t>
+          <t>Talk where the music isn't. Gym speakers play licensed music, your mic will pick it up, and TikTok and Instagram scan audio automatically. A muted talking video is a dead video. So: record talking parts in your car in the gym lot or a music-free corner, and use the gym floor for silent B-roll. Turn on TikTok's 'Music copyright check' on the posting page. A $20-40 tripod with a Bluetooth remote is worth buying.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>TIMING</t>
+          <t>POSTING STACK (phone-only)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>First post (Wed): TikTok at 7:30 AM ET, which leaves 45 minutes after the gym to edit and proof captions. From Thursday: TikTok at 7:00 AM ET, Instagram Reels the next morning at 8:00 AM ET (in line with Hootsuite's morning window and Hopper's 7-8 AM Reels finding). Week 3: test one evening slot (6-8 PM, Metricool's TikTok study). After about 3 weeks of posts, switch to Metricool's personalized 'Best times' for your own audience.</t>
+          <t>Write/tighten scripts in the Claude app → film at your gym on a $20-40 tripod with a noise-cancelling clip mic (DJI Mic Mini class, ~$79 on sale) → edit + auto-captions in CapCut (TikTok master) → re-caption/finish the Instagram version in Edits (Instagram's free editor, no watermark) → schedule/auto-publish both through Metricool (already connected) → check TikTok Creative Center and your own For You page 10 min a day for trends. No AI faces, AI voices, or AI eye-contact fixes. Raw stays raw.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>FIRST POST</t>
+          <t>SEQUENCE</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Post Script B ('The Acronym') first: it has the strongest 1-second hook and explains the channel. Post Script C ('5:40 AM') second and Script A ('The Parking Lot') third. Film all three Wednesday morning, and pin all three on TikTok (it allows 3 pinned videos). Captions are burned into every video.</t>
+          <t>TikTok first, every time. Repurpose to Instagram Reels about 24 hours later with a clean export (no TikTok watermark) and fresh captions. TikTok's For You feed ranks on content signals, not follower count, so a zero-follower account can reach people on day one. Instagram rewards originality and 'sends' (shares by DM), so post a native, clean upload rather than a repost.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>CONTENT PILLARS</t>
+          <t>TIMING</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>1) 5AM Brain. 2) AI External Brain (incl. prompting as a skill and the will-NOT list). 3) Late-Diagnosis Log. 4) AI for Your Family. 5) ADHD Dad in the Wild. 6) NotebookLM (personal use cases, not tutorials). 15 starter ideas each, plus 3 freshly researched ideas per pillar in every Sunday doc.</t>
+          <t>First post (Wed): TikTok at 7:30 AM ET, which leaves 45 minutes after the gym to edit and proof captions. From Thursday: TikTok at 7:00 AM ET, Instagram Reels the next morning at 8:00 AM ET (in line with Hootsuite's morning window and Hopper's 7-8 AM Reels finding). Week 3: test one evening slot (6-8 PM, Metricool's TikTok study). After about 3 weeks of posts, switch to Metricool's personalized 'Best times' for your own audience.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>FIRST POST</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>First post is a teaser (Wed Oct 21): a real moment, no explanation. Script B ('The Acronym') moves to reveal day, Wed Nov 4, with Script A ('The Parking Lot') on Thu Nov 5 and Script C ('5:40 AM') on Fri Nov 6. Pin all three after the reveal (TikTok allows 3 pinned videos). Captions are burned into every video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>CONTENT PILLARS</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>1) 5AM Brain. 2) AI External Brain (incl. prompting as a skill and the will-NOT list). 3) Late-Diagnosis Log. 4) AI for Your Family. 5) ADHD Dad in the Wild. 6) NotebookLM (personal use cases, not tutorials). 15 starter ideas each, plus 3 freshly researched ideas per pillar in every Sunday doc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
           <t>WHAT I COULDN'T VERIFY</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>The sandbox only allows web search, so I couldn't directly query USPTO, domain registries, or TikTok/Instagram profile pages. Trademark findings come from indexed USPTO-data mirrors (Justia, Trademarkia, uspto.report, TTABVUE). Handle and domain status is 'no existing use found', not 'confirmed available'. Instagram reach penalties for muted audio come from third-party guides; Meta hasn't confirmed them. None of this is legal advice. Before you file a federal application, get a 1-hour clearance review from a trademark attorney.</t>
         </is>
@@ -617,6 +642,639 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="47" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TikTok first, Instagram the next morning. Reply to every comment within the first 60 minutes. Teasers follow the rules in Launch Phases; each slot gives the story shape, and you film your real version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Time (ET)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tue Oct 20</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Set the teaser-phase bios (see Bio); film teasers 1-3</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>If Scripts B, C or A are already live, see Assumptions 37.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Wed Oct 21</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 1: The empty gym before sunrise: what your mornings look like now. Don't say why.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Pin it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thu Oct 22</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 2: A moment your son read something he couldn't before (with your wife's OK). Don't say what helped.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Fri Oct 23</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 3: Keys on the hook, found first try. The result, played completely straight.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Sat Oct 24</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 4: The email or task you'd been avoiding for weeks: sent. Show the 'sent' screen with private info covered.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Sunday: batch-film the next teasers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Mon Oct 26</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 5: A conversation a couple of months ago changed how you run your day. Say that much and stop.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Tue Oct 27</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 6: Two seconds of audio that says your name, then your face reacting. Cut before you explain.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Wed Oct 28</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 7: What your wife noticed changed first (only with her OK). Her words, not the reason.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Thu Oct 29</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 8: The family calendar on the fridge that's actually up to date this week.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Fri Oct 30</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 9: Halloween costume sorted before Oct 30 (post Thu Oct 29). Deadpan.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Sat Oct 31</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 10: A week of 5 AM sessions in 10 seconds. One line: 'Still going.'</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Also check: 3+ posts with 'how?' comments? Then reveal Mon Nov 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Mon Nov 2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 11: Things you don't forget anymore, as an on-screen list. No explanation.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Tue Nov 3</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Teaser 12: The day before the reveal: 'Tomorrow I'll tell you what changed. Read my name slowly.'</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>1 · Tease</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Wed Nov 4</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Script B: 'The Acronym'</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>2 · Reveal</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Switch both bios to the reveal versions first. Post natively with 'Music copyright check' on; reply for the first hour. Pin it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Thu Nov 5</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Script A: 'The Parking Lot'</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>2 · Reveal</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Pin it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Fri Nov 6</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Script C: '5:40 AM'</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>2 · Reveal</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Pin it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Sat Nov 7</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Reply video to the best 'how?' comment from the teaser phase</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>2 · Reveal</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>TikTok's 'reply with video' button</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Mon Nov 9</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>7:00 AM ET</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>AI External Brain: 'The prompt I use when I can't start anything'</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>3 · Rhythm</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Weekly pillar rhythm starts. Put the prompt in the caption so people can copy it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Every day</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>8:00 AM ET (next day)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Instagram Reel</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Yesterday's TikTok (watermark-free export, Edits captions)</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Via Metricool, or in-app if not connected yet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -914,7 +1572,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -969,7 +1627,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Recommended order: B first, C second, A third. Pin all three.</t>
+          <t>These three are the reveal-week videos: B on Wed Nov 4, A on Thu Nov 5, C on Fri Nov 6. Don't post them during the teaser phase (see Launch Phases). Pin all three after the reveal.</t>
         </is>
       </c>
     </row>
@@ -1589,17 +2247,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
     <col width="53" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
@@ -1647,22 +2305,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Name (teaser phase, to Nov 3)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>ADHD Dad | AI Dad Healthy Dad</t>
+          <t>AI Dad Healthy Dad</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>29 of 30</t>
+          <t>18 of 30</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Searchable. 'ADHD Dad' first so it shows in search previews.</t>
+          <t>Leaves out 'ADHD Dad' until the reveal. The name itself is the clue: the initials spell ADHD.</t>
         </is>
       </c>
     </row>
@@ -1674,20 +2332,25 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Username</t>
+          <t>Bio (teaser phase, to Nov 3)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>@aidadhealthydad</t>
+          <t>Dad · 5AM gym · results first
+The how: Nov 4 · DMs open</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>16 of 24</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
+          <t>55 of 80</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Promises results now and the how on a date, without saying what the how is.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1697,75 +2360,75 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>ADHD Dad | AI Dad Healthy Dad</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>29 of 30</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>From Nov 4 (reveal). Searchable: 'ADHD Dad' first so it shows in search previews.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>@aidadhealthydad</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>16 of 24</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
           <t>Bio</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Late-diagnosed ADHD dad · 5AM gym
 AI = my external brain · DMs open</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>67 of 80</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Each term comes from this sheet's trend list (late-diagnosed, ADHD dad, 5AM, external brain). Soft CTA = 'DMs open'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>AI Dad Healthy Dad | Late-Diagnosed ADHD Dad</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>44 of 64</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Instagram searches the name field hardest, so it carries the top trend term. Instagram limits name changes (twice in 14 days), so set it once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Username</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>@aidadhealthydad</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>16 of 30</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>From Nov 4 (reveal). Each term comes from this sheet's trend list (late-diagnosed, ADHD dad, 5AM, external brain). Soft CTA = 'DMs open'.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1775,10 +2438,117 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
+          <t>Name (teaser phase, to Nov 3)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>AI Dad Healthy Dad</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>18 of 64</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Instagram allows 2 name changes in 14 days: this one now, the reveal name on Nov 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Bio (teaser phase, to Nov 3)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Dad · 5AM gym before the house wakes up
+A lot changed in about a month
+Results first. The how: Nov 4
+DMs open</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>109 of 150</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Same idea as TikTok, with room for one more line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>AI Dad Healthy Dad | Late-Diagnosed ADHD Dad</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>44 of 64</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Instagram searches the name field hardest, so it carries the top trend term. Instagram limits name changes (twice in 14 days), so set it once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>@aidadhealthydad</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>16 of 30</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
           <t>Bio</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Late-diagnosed ADHD dad
 5AM gym before the house wakes up
@@ -1787,46 +2557,46 @@
 DMs open</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>146 of 150</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Lines 1-3 are search terms. Line 4 is the trust signal: the misinformation-backlash trend, and 'AI Dad' shouldn't read as an AI persona. Category: Digital creator. Add the link once aidadhealthydad.com is live.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>From Nov 4 (reveal). Lines 1-3 are search terms. Line 4 is the trust signal: the misinformation-backlash trend, and 'AI Dad' shouldn't read as an AI persona. Category: Digital creator. Add the link once aidadhealthydad.com is live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Pinned / Highlights</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Pin Scripts B, C, A on TikTok. Instagram Highlights: 'Start Here', '5AM Gym', 'AI Prompts', 'Diagnosis Log'.</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>From Nov 4: pin Scripts B, A, C on TikTok. Instagram Highlights: 'Start Here', '5AM Gym', 'AI Prompts', 'Diagnosis Log'.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1845,7 +2615,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Weekly rhythm: Mon AI External Brain · Tue AI for Your Family · Wed 5AM Brain · Thu ADHD Dad in the Wild · Fri Late-Diagnosis Log · Sat NotebookLM + reply-to-comment video · Sun batch-film (the weekly ideas doc lands at 5 AM ET). 6 pillars × 15 starter ideas; fresh researched ideas arrive every Sunday. Ideas are story shapes: you supply the real story live.</t>
+          <t>From Mon Nov 9 (after the teaser phase and reveal week; see Launch Phases). Weekly rhythm: Mon AI External Brain · Tue AI for Your Family · Wed 5AM Brain · Thu ADHD Dad in the Wild · Fri Late-Diagnosis Log · Sat NotebookLM + reply-to-comment video · Sun batch-film (the weekly ideas doc lands at 5 AM ET). 6 pillars × 15 starter ideas; fresh researched ideas arrive every Sunday. Ideas are story shapes: you supply the real story live.</t>
         </is>
       </c>
     </row>
@@ -1940,7 +2710,7 @@
 3) The school flyer trick: photo of the flyer, AI turns it into reminders. Save: the 3-step workflow.
 4) The worry sort: voice-memo everything on my mind, and AI sorts it into today / this week / not mine. Save: the sorting prompt.
 5) I asked AI if my channel name was trademarked: what it found, and what it said I still had to check myself. Save: the 'verify it yourself' list.
-6) AI built me a spreadsheet with 864 rows. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
+6) AI built me a spreadsheet with 973 rows. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
 7) The 'am I sliding?' check-in: one sentence to AI when the old pattern starts, and it asks me 3 questions back. Save: the 3 questions.
 8) 'Remind me later' → a real calendar event in 10 seconds, hands-free. Save: the dictation phrasing that works.
 9) What I will NOT use AI for: talking to my kids, apologizing to my wife, health decisions. Save: my human-only list.
@@ -2154,13 +2924,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2778,7 +3548,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>The weekly doc is a new Google Doc every Sunday at 5 AM ET in your Drive, titled 'AI Dad Weekly Ideas · Week of ...'. It comes from a routine you set up yourself at claude.ai/code/routines (Sundays 4:52 AM ET), using the prompt in docs/weekly_routine_prompt.md. It never edits this sheet.</t>
+          <t>The weekly doc is a new Google Doc every Sunday at 5 AM ET in your Drive, titled 'AI Dad Weekly Scripts · Week of ...'. It comes from a routine you set up yourself at claude.ai/code/routines (Sundays 4:52 AM ET), using the prompt in docs/weekly_routine_prompt.md. It never edits this sheet.</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2801,6 +3571,57 @@
       <c r="C39" s="3" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>The teaser plan assumes Scripts B, C and A haven't been posted yet (the old calendar had them on Oct 14-16).</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>If any are live, the reveal already happened on that account: either make them private before teaser 1, or skip Phase 1 and keep the normal rhythm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1 length (2 weeks, 12 posts) is a judgment call. No study measures teaser length for new accounts; it rests on TikTok's description of how videos get matched, new-account guides (test phase of about 10-20 videos, traction about 90 days) and practitioner teaser advice (2-3 weeks). Those numbers come from search summaries, not pages I opened.</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Use the 'reveal early' rule, and don't stretch Phase 1 for low views.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Oct 19: three 'Weekly Scripts · Week of Oct 19' docs came from three separate manual runs of the routine on Oct 18, each creating a fresh doc. The 3:00 PM one was kept; the other two and the superseded Oct 18 'Weekly Ideas' doc went to Drive's trash. The routine now checks Drive first and won't make a second doc for the same week.</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>To deliberately regenerate a week, run it with the word REDO; the old doc is renamed '(old)', never deleted.</t>
         </is>
       </c>
     </row>
@@ -2809,17 +3630,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="51" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -4176,15 +4997,134 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
+          <t>Launch phases</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>TikTok newsroom: how TikTok recommends videos #ForYou</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>https://newsroom.tiktok.com/en-us/how-tiktok-recommends-videos-for-you/</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Launch phases</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Buffer: how often to post on TikTok (11M+ posts, Oct 2025)</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>https://buffer.com/resources/how-often-should-you-post-on-tiktok/</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Launch phases</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Socialync: TikTok algorithm tips for new accounts 2026 (test phase, ~video 15-30 breakout)</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.socialync.io/blog/tiktok-algorithm-tips-new-accounts-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Launch phases</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>ContentLoop: new-account traction ~90 days (growth guide)</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>https://contentloop.it.com/?p=1411</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Launch phases</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>VBJ column 'Tease, please': teaser 2-3 weeks before launch</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.vbjusa.com/opinion/columns/marketing-strategic-communication-column/column-tease-please/</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Launch phases</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>ZoomSphere: teaser timelines past 2 weeks lose people (unsourced claim)</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zoomsphere.com/blog/is-your-teaser-a-hook-or-just-a-delay-tactic</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Launch phases</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Descript: the curiosity gap (open it, then close it)</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.descript.com/blog/article/the-youtubers-guide-to-the-curiosity-gap-how-to-keep-your-audiences-interest</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
           <t>Filming</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>PureGym filming rule (STV News)</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C89" s="3" t="inlineStr">
         <is>
           <t>https://news.stv.tv/world/gym-fluencers-urged-to-stop-filming-in-public-amid-privacy-concerns</t>
         </is>
@@ -6427,469 +7367,205 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="57" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TikTok first, Instagram next day. Reply to every comment within the first 60 minutes of each post. Launch week runs the three intro scripts Wed-Fri; the weekly rhythm in Content Pillars starts Monday.</t>
+          <t>Phase 1 teases real-life moments and results without explaining the mechanism. Phase 2 reveals it: the AI-and-ADHD angle. The phase length below was chosen from research on new accounts (sources in the Sources section, marked 'Launch phases'). No study measures teaser length directly, so the call is reasoned from what is known.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Time (ET)</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Post</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Pillar</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>Why</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Tue Oct 13</t>
+          <t>Phase 1: teaser length</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>2 weeks, 12 posts: Wed Oct 21 to Tue Nov 3, Monday to Saturday at 7:00 AM ET. Sundays are for filming.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Claim handles + domain, connect Metricool, set bios, pack the filming kit</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Read each script's Detail check row tonight and swap anything that isn't true for you.</t>
+          <t>Short on purpose. A brand-new account has no audience to keep in suspense: most viewers see one video, not the series. TikTok matches videos to viewers using captions, sounds, hashtags and what people watch (TikTok newsroom), so every week without 'ADHD dad' in the words is a week the app can't tell who your videos are for. Practitioner guidance on teasers says 2-3 weeks before interest wears out; one curiosity-marketing piece says people check out after 2 weeks. I took the low end.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Wed Oct 14</t>
+          <t>Why not shorter</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>5:30-6:45 AM ET</t>
+          <t>Not 1 week (6 posts).</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Film at the gym: Script A in the car first, then B and C (talking parts in a music-free spot, B-roll on the floor)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Film all three now; post only B today.</t>
+          <t>New-account guides describe roughly the first 10-20 videos as the test phase where the app is still working out who to show you to (a creator rule of thumb, not TikTok data). 12 teasers sit inside that window and give enough posts for a returning viewer to notice a pattern before the reveal lands on video 13.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Wed Oct 14</t>
+          <t>Reveal early if</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>7:30 AM ET</t>
+          <t>After at least 6 teasers, if 3 or more posts get comments asking how or why, reveal on the next posting day.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Script B: 'The Acronym'</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Intro</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Moved from 7:00 to leave 45 min to edit and proof captions. Post natively in the TikTok app with 'Music copyright check' on; reply for the first hour. Pin it.</t>
+          <t>Those comments are the curiosity the teaser phase exists to create. Once it shows up, cashing it in beats making people wait.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Thu Oct 15</t>
+          <t>Never stretch it</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>7:00 AM ET</t>
+          <t>Don't extend Phase 1 because views are low.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Script C: '5:40 AM'</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>5AM Brain</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Pin it.</t>
+          <t>Low views in weeks 1-2 are normal for any new account: growth guides put meaningful traction at about 90 days of consistent posting. Keeping the mystery longer won't fix that, and it keeps your search words hidden.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Thu Oct 15</t>
+          <t>Phase 2: reveal</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>8:00 AM ET</t>
+          <t>Wed Nov 4 Script B ('The Acronym') · Thu Nov 5 Script A ('The Parking Lot') · Fri Nov 6 Script C ('5:40 AM') · Sat Nov 7 reply video to the best 'how?' comment from Phase 1.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Instagram Reel</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Script B (watermark-free export, Edits captions)</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Intro</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Via Metricool, or in-app if not connected yet</t>
+          <t>The account name is already the clue (the initials spell ADHD), so B pays it off. Switch both bios to the reveal versions the morning of Nov 4. Pin B, A and C.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Fri Oct 16</t>
+          <t>Phase 3: normal rhythm</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>7:00 AM ET</t>
+          <t>From Mon Nov 9: the 6-pillar weekly rhythm in Content Pillars.</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Script A: 'The Parking Lot'</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Late-Diagnosis Log</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Pin it.</t>
+          <t>Each teaser maps to a pillar, so every Phase 1 moment gets a full 'here's how' video later.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Fri Oct 16</t>
+          <t>Teaser rules</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>8:00 AM ET</t>
+          <t>Show a real moment and a real result. Say what changed, never why. No 'ADHD', 'AI', 'diagnosis' or app names in the video, captions, on-screen text or hashtags. End each teaser with a line like 'More on that soon.'</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Instagram Reel</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Script C</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>5AM Brain</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Metricool</t>
+          <t>The mystery has to come from the result, not from withholding the point: each video still has to be worth watching on its own.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Sat Oct 17</t>
+          <t>Teaser honesty</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>7:00 AM ET</t>
+          <t>Only real results, no invented timelines. If someone asks how, reply: 'Telling the whole story on Nov 4.' Never deny it or make up a different reason.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Reply-to-comment video (best question from Wed-Fri)</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Comment Answers</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>TikTok's 'reply with video' button</t>
+          <t>Teasing builds trust only if the reveal matches the hints.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Sat Oct 17</t>
+          <t>Hard boundary (still)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>8:00 AM ET</t>
+          <t>Teasers never hint at the specific habit. 'Something changed' is about mornings, family and focus, nothing more.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Instagram Reel</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Script A</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Late-Diagnosis Log</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Metricool</t>
+          <t>Per CLAUDE.md. Vague mystery copy can read as a hint, so keep every teaser on a visible result.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Sat Oct 17</t>
+          <t>Teaser hashtags</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>9:00 AM ET</t>
+          <t>Results and dad tags only, e.g. #dadsoftiktok #dadlife #5amclub #morningroutine. Re-check them weekly.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Instagram carousel</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Carousel: 'The 3 calls I make between sets' (from Script C)</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>5AM Brain</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Saveable checklist</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Sun Oct 18</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>5:00 AM ET</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Weekly ideas doc lands; batch-film 3-4 videos</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Pick from the doc and the starter lists</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Mon Oct 19</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>7:00 AM ET</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>AI External Brain #1: 'The prompt I use when I can't start anything'</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>AI External Brain</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Put the prompt in the caption so people can copy it</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Tue Oct 20</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>7:00 AM ET</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>AI for Your Family: 'The reading podcast'</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>AI for Your Family</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Flagship story. Hook from the weekly doc; you tell it live, with your wife's OK.</t>
+          <t>Keeps the mechanism hidden while still giving the app words to match you on.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Launch plan: fix teaser order, reveal-day labels, IG name note
Rebuilt deliverables after write to the Google Sheet (verified 974/974
rows). README lists the routine prompt file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqY8QbXMfegJWDBpeB6XE4
</commit_message>
<xml_diff>
--- a/deliverables/AI_Dad_Launch_Plan.xlsx
+++ b/deliverables/AI_Dad_Launch_Plan.xlsx
@@ -951,7 +951,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Teaser 8: The family calendar on the fridge that's actually up to date this week.</t>
+          <t>Teaser 8: Halloween costume sorted before Oct 30. Deadpan.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Teaser 9: Halloween costume sorted before Oct 30 (post Thu Oct 29). Deadpan.</t>
+          <t>Teaser 9: The family calendar on the fridge that's actually up to date this week.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Say 'ADHD dad' in the first 3 seconds, put it in the first on-screen text, and in the first line of the caption.</t>
+          <t>From the reveal on (not in teasers): say 'ADHD dad' in the first 3 seconds, put it in the first on-screen text, and in the first line of the caption.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (POST FIRST)</t>
+          <t>B: The Acronym (REVEAL DAY)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1698,7 +1698,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (POST FIRST)</t>
+          <t>B: The Acronym (REVEAL DAY)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1730,7 +1730,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (POST FIRST)</t>
+          <t>B: The Acronym (REVEAL DAY)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1762,7 +1762,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (POST FIRST)</t>
+          <t>B: The Acronym (REVEAL DAY)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1794,7 +1794,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (POST FIRST)</t>
+          <t>B: The Acronym (REVEAL DAY)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (POST FIRST)</t>
+          <t>B: The Acronym (REVEAL DAY)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Instagram searches the name field hardest, so it carries the top trend term. Instagram limits name changes (twice in 14 days), so set it once.</t>
+          <t>From Nov 4 (reveal). Instagram searches the name field hardest, so it carries the top trend term. This is the second of the two name changes Instagram allows in 14 days, so get it right first time.</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2710,7 @@
 3) The school flyer trick: photo of the flyer, AI turns it into reminders. Save: the 3-step workflow.
 4) The worry sort: voice-memo everything on my mind, and AI sorts it into today / this week / not mine. Save: the sorting prompt.
 5) I asked AI if my channel name was trademarked: what it found, and what it said I still had to check myself. Save: the 'verify it yourself' list.
-6) AI built me a spreadsheet with 973 rows. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
+6) AI built me a spreadsheet with 974 rows. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
 7) The 'am I sliding?' check-in: one sentence to AI when the old pattern starts, and it asks me 3 questions back. Save: the 3 questions.
 8) 'Remind me later' → a real calendar event in 10 seconds, hands-free. Save: the dictation phrasing that works.
 9) What I will NOT use AI for: talking to my kids, apologizing to my wife, health decisions. Save: my human-only list.

</xml_diff>

<commit_message>
Launch: B already live, one secrecy rule, 6-post tease, reveal Oct 28
- Script B is marked as live on TikTok (Instagram Wed Oct 21)
- Same rule on both platforms: ADHD and "I use AI" are open; specific
  tools and the workflow stay hidden until the reveal
- Phase 1 is now 6 teasers (Oct 21-27); reveal Wed Oct 28, A Thu,
  C Fri, reply video Sat; pillar rhythm from Mon Nov 2
- Teaser bios, calendar, assumptions, checker, CLAUDE.md and the
  weekly routine prompt updated to match

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqY8QbXMfegJWDBpeB6XE4
</commit_message>
<xml_diff>
--- a/deliverables/AI_Dad_Launch_Plan.xlsx
+++ b/deliverables/AI_Dad_Launch_Plan.xlsx
@@ -457,7 +457,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Dad ___ Dad: launch plan. Research done 2026-10-13; updated Oct 19: tease first, reveal on Wed Nov 4. First teaser post: Wednesday, Oct 21, 2026, morning.</t>
+          <t>AI Dad ___ Dad: launch plan. Research done 2026-10-13; updated Oct 19: 6 teaser posts, reveal on Wed Oct 28. First teaser post: Wednesday, Oct 21, 2026, morning.</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>(1) Launch is now tease-then-reveal. For the first 2 weeks (12 posts, Wed Oct 21 to Tue Nov 3) you show real moments and results and never explain the why: no 'ADHD', no 'AI'. Wed Nov 4 is the reveal (Script B, 'The Acronym'). See the new 'Launch Phases' section for why 2 weeks. (2) The calendar is now the 'Launch Calendar'. (3) New teaser-phase bios. (4) The weekly routine can no longer create a second doc for the same week.</t>
+          <t>(1) Launch is tease-then-reveal: 6 teaser posts, Wed Oct 21 to Tue Oct 27, then the reveal on Wed Oct 28. (2) One rule on TikTok and Instagram: ADHD and 'I use AI' are fine to say; only the specific tools and how you use them stay hidden until Oct 28. (3) Script B ('The Acronym') is already live on TikTok, and it fits that rule. (4) The calendar is now the 'Launch Calendar'. (5) The weekly routine can no longer create a second doc for the same week.</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Weeks 1-2: results without the how. Week 3: the reveal. Each teaser must work on its own (a real moment, a real result, a clean ending) because a brand-new account's viewers mostly see one video, not the series. If people keep asking 'how?' in the comments, reveal early (rule in Launch Phases).</t>
+          <t>Posts 1-6: real results, and the fact that AI is behind them, but never which tools or how. Oct 28: the reveal, showing the actual setup. Each teaser must work on its own (a real moment, a real result, a clean ending) because a brand-new account's viewers mostly see one video, not the series.</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>First post is a teaser (Wed Oct 21): a real moment, no explanation. Script B ('The Acronym') moves to reveal day, Wed Nov 4, with Script A ('The Parking Lot') on Thu Nov 5 and Script C ('5:40 AM') on Fri Nov 6. Pin all three after the reveal (TikTok allows 3 pinned videos). Captions are burned into every video.</t>
+          <t>Script B ('The Acronym') is already live on TikTok: keep it pinned, and post it on Instagram Wed Oct 21. First teaser: Wed Oct 21. The reveal video (Wed Oct 28) shows the actual tools; Script A ('The Parking Lot') follows on Thu Oct 29 and Script C ('5:40 AM') on Fri Oct 30. Pin A and C next to B (TikTok allows 3 pinned videos). Captions are burned into every video.</t>
         </is>
       </c>
     </row>
@@ -647,13 +647,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="47" customWidth="1" min="6" max="6"/>
   </cols>
@@ -700,99 +700,99 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Tue Oct 20</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Set the teaser-phase bios (see Bio); film teasers 1-3</t>
+          <t>Script B: 'The Acronym'</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>If Scripts B, C or A are already live, see Assumptions 37.</t>
+          <t>Already live. Keep it pinned.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Wed Oct 21</t>
+          <t>Tue Oct 20</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>7:00 AM ET</t>
+          <t>Evening</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Teaser 1: The empty gym before sunrise: what your mornings look like now. Don't say why.</t>
+          <t>Set the names and teaser-phase bios (see Bio); film teasers 1-3</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1 · Tease</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Pin it.</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Thu Oct 22</t>
+          <t>Wed Oct 21</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>7:00 AM ET</t>
+          <t>8:00 AM ET</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram Reel</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Teaser 2: A moment your son read something he couldn't before (with your wife's OK). Don't say what helped.</t>
+          <t>Script B: 'The Acronym' (watermark-free export, Edits captions)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1 · Tease</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
+          <t>Intro</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Its first Instagram post.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Fri Oct 23</t>
+          <t>Wed Oct 21</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Teaser 3: Keys on the hook, found first try. The result, played completely straight.</t>
+          <t>Teaser 1: The empty gym before sunrise: what ADHD mornings look like now that AI holds my to-do list. Don't show how.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -820,7 +820,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Sat Oct 24</t>
+          <t>Thu Oct 22</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Teaser 4: The email or task you'd been avoiding for weeks: sent. Show the 'sent' screen with private info covered.</t>
+          <t>Teaser 2: A moment your son read something he couldn't before (with your wife's OK). Say AI helped; don't say which tool.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -843,16 +843,12 @@
           <t>1 · Tease</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Sunday: batch-film the next teasers.</t>
-        </is>
-      </c>
+      <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Mon Oct 26</t>
+          <t>Fri Oct 23</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -867,7 +863,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Teaser 5: A conversation a couple of months ago changed how you run your day. Say that much and stop.</t>
+          <t>Teaser 3: Keys on the hook, found first try: 'Same ADHD brain. New system.' No screens.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -880,7 +876,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Tue Oct 27</t>
+          <t>Sat Oct 24</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -895,7 +891,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Teaser 6: Two seconds of audio that says your name, then your face reacting. Cut before you explain.</t>
+          <t>Teaser 4: The email you'd avoided for weeks, sent in under a minute. Show only the 'sent' screen, private info covered.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -903,12 +899,16 @@
           <t>1 · Tease</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Sunday: film the reveal video and Scripts A and C.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Wed Oct 28</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Teaser 7: What your wife noticed changed first (only with her OK). Her words, not the reason.</t>
+          <t>Teaser 5: Two seconds of a podcast that says your name, then your face reacting: 'An AI made this about me.' Cut there.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -931,12 +931,16 @@
           <t>1 · Tease</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Check: 2+ posts with 'which app?' comments? Then reveal tomorrow.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Thu Oct 29</t>
+          <t>Tue Oct 27</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -951,7 +955,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Teaser 8: Halloween costume sorted before Oct 30. Deadpan.</t>
+          <t>Teaser 6: Halloween costume sorted early, then: 'Tomorrow I'll show you the exact setup.'</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -964,7 +968,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Fri Oct 30</t>
+          <t>Wed Oct 28</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -979,20 +983,24 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Teaser 9: The family calendar on the fridge that's actually up to date this week.</t>
+          <t>Reveal: the actual tools and one real example of each, on screen</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>1 · Tease</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr"/>
+          <t>2 · Reveal</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Switch both bios to the reveal versions first. Post natively with 'Music copyright check' on; reply for the first hour. Pin it.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Sat Oct 31</t>
+          <t>Thu Oct 29</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1007,24 +1015,24 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Teaser 10: A week of 5 AM sessions in 10 seconds. One line: 'Still going.'</t>
+          <t>Script A: 'The Parking Lot'</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>1 · Tease</t>
+          <t>2 · Reveal</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Also check: 3+ posts with 'how?' comments? Then reveal Mon Nov 2.</t>
+          <t>Pin it.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Mon Nov 2</t>
+          <t>Fri Oct 30</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1039,20 +1047,24 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Teaser 11: Things you don't forget anymore, as an on-screen list. No explanation.</t>
+          <t>Script C: '5:40 AM'</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>1 · Tease</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr"/>
+          <t>2 · Reveal</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Pin it (TikTok keeps 3 pins: B, A, C).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Tue Nov 3</t>
+          <t>Sat Oct 31</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1067,20 +1079,24 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Teaser 12: The day before the reveal: 'Tomorrow I'll tell you what changed. Read my name slowly.'</t>
+          <t>Reply video to the best 'which app?' comment</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1 · Tease</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr"/>
+          <t>2 · Reveal</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>TikTok's 'reply with video' button</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Wed Nov 4</t>
+          <t>Mon Nov 2</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1095,175 +1111,47 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Script B: 'The Acronym'</t>
+          <t>AI External Brain: 'The prompt I use when I can't start anything'</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>2 · Reveal</t>
+          <t>3 · Rhythm</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Switch both bios to the reveal versions first. Post natively with 'Music copyright check' on; reply for the first hour. Pin it.</t>
+          <t>Weekly pillar rhythm starts. Put the prompt in the caption so people can copy it.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Thu Nov 5</t>
+          <t>Every day</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>7:00 AM ET</t>
+          <t>8:00 AM ET (next day)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram Reel</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Script A: 'The Parking Lot'</t>
+          <t>Yesterday's TikTok (watermark-free export, Edits captions)</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>2 · Reveal</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Pin it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Fri Nov 6</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>7:00 AM ET</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Script C: '5:40 AM'</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>2 · Reveal</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Pin it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Sat Nov 7</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>7:00 AM ET</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Reply video to the best 'how?' comment from the teaser phase</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>2 · Reveal</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>TikTok's 'reply with video' button</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Mon Nov 9</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>7:00 AM ET</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>AI External Brain: 'The prompt I use when I can't start anything'</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>3 · Rhythm</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Weekly pillar rhythm starts. Put the prompt in the caption so people can copy it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Every day</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>8:00 AM ET (next day)</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Instagram Reel</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Yesterday's TikTok (watermark-free export, Edits captions)</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Via Metricool, or in-app if not connected yet</t>
         </is>
@@ -1558,7 +1446,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>From the reveal on (not in teasers): say 'ADHD dad' in the first 3 seconds, put it in the first on-screen text, and in the first line of the caption.</t>
+          <t>Say 'ADHD dad' in the first 3 seconds, put it in the first on-screen text, and in the first line of the caption.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1581,7 +1469,7 @@
   <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="68" customWidth="1" min="4" max="4"/>
@@ -1627,7 +1515,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>These three are the reveal-week videos: B on Wed Nov 4, A on Thu Nov 5, C on Fri Nov 6. Don't post them during the teaser phase (see Launch Phases). Pin all three after the reveal.</t>
+          <t>B is already live on TikTok (it goes on Instagram Wed Oct 21). A and C go out after the reveal: Thu Oct 29 and Fri Oct 30. Pin all three.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1554,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (REVEAL DAY)</t>
+          <t>B: The Acronym (LIVE ON TIKTOK)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1698,7 +1586,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (REVEAL DAY)</t>
+          <t>B: The Acronym (LIVE ON TIKTOK)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1730,7 +1618,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (REVEAL DAY)</t>
+          <t>B: The Acronym (LIVE ON TIKTOK)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1762,7 +1650,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (REVEAL DAY)</t>
+          <t>B: The Acronym (LIVE ON TIKTOK)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1794,7 +1682,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (REVEAL DAY)</t>
+          <t>B: The Acronym (LIVE ON TIKTOK)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1826,7 +1714,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>B: The Acronym (REVEAL DAY)</t>
+          <t>B: The Acronym (LIVE ON TIKTOK)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2253,11 +2141,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="53" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
@@ -2305,22 +2193,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Name (teaser phase, to Nov 3)</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>AI Dad Healthy Dad</t>
+          <t>ADHD Dad | AI Dad Healthy Dad</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>18 of 30</t>
+          <t>29 of 30</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Leaves out 'ADHD Dad' until the reveal. The name itself is the clue: the initials spell ADHD.</t>
+          <t>Set it now. Searchable: 'ADHD Dad' first so it shows in search previews.</t>
         </is>
       </c>
     </row>
@@ -2332,25 +2220,20 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Bio (teaser phase, to Nov 3)</t>
+          <t>Username</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Dad · 5AM gym · results first
-The how: Nov 4 · DMs open</t>
+          <t>@aidadhealthydad</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>55 of 80</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Promises results now and the how on a date, without saying what the how is.</t>
-        </is>
-      </c>
+          <t>16 of 24</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2360,22 +2243,23 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Bio (teaser, to Oct 27)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>ADHD Dad | AI Dad Healthy Dad</t>
+          <t>Late-diagnosed ADHD dad · 5AM gym
+AI changed my days. The how: Oct 28</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>29 of 30</t>
+          <t>69 of 80</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>From Nov 4 (reveal). Searchable: 'ADHD Dad' first so it shows in search previews.</t>
+          <t>Says ADHD and AI, promises the how on a date, names no tools.</t>
         </is>
       </c>
     </row>
@@ -2387,46 +2271,50 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Username</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>@aidadhealthydad</t>
+          <t>Late-diagnosed ADHD dad · 5AM gym
+AI = my external brain · DMs open</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>16 of 24</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
+          <t>67 of 80</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>From Oct 28 (reveal). Each term comes from this sheet's trend list (late-diagnosed, ADHD dad, 5AM, external brain). Soft CTA = 'DMs open'.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Late-diagnosed ADHD dad · 5AM gym
-AI = my external brain · DMs open</t>
+          <t>AI Dad Healthy Dad | Late-Diagnosed ADHD Dad</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>67 of 80</t>
+          <t>44 of 64</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>From Nov 4 (reveal). Each term comes from this sheet's trend list (late-diagnosed, ADHD dad, 5AM, external brain). Soft CTA = 'DMs open'.</t>
+          <t>Set it now. Instagram searches the name field hardest, so it carries the top trend term. Instagram limits name changes (twice in 14 days), so set it once.</t>
         </is>
       </c>
     </row>
@@ -2438,24 +2326,20 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Name (teaser phase, to Nov 3)</t>
+          <t>Username</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>AI Dad Healthy Dad</t>
+          <t>@aidadhealthydad</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>18 of 64</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Instagram allows 2 name changes in 14 days: this one now, the reveal name on Nov 4.</t>
-        </is>
-      </c>
+          <t>16 of 30</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2465,25 +2349,26 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Bio (teaser phase, to Nov 3)</t>
+          <t>Bio (teaser, to Oct 27)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Dad · 5AM gym before the house wakes up
-A lot changed in about a month
-Results first. The how: Nov 4
+          <t>Late-diagnosed ADHD dad
+5AM gym before the house wakes up
+AI rebuilt my days. The how: Oct 28
+Real dad, no AI faces · not medical advice
 DMs open</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>109 of 150</t>
+          <t>145 of 150</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Same idea as TikTok, with room for one more line.</t>
+          <t>Same idea as TikTok.</t>
         </is>
       </c>
     </row>
@@ -2495,60 +2380,10 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>AI Dad Healthy Dad | Late-Diagnosed ADHD Dad</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>44 of 64</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>From Nov 4 (reveal). Instagram searches the name field hardest, so it carries the top trend term. This is the second of the two name changes Instagram allows in 14 days, so get it right first time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Username</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>@aidadhealthydad</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>16 of 30</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Bio</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Late-diagnosed ADHD dad
 5AM gym before the house wakes up
@@ -2557,39 +2392,39 @@
 DMs open</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>146 of 150</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>From Nov 4 (reveal). Lines 1-3 are search terms. Line 4 is the trust signal: the misinformation-backlash trend, and 'AI Dad' shouldn't read as an AI persona. Category: Digital creator. Add the link once aidadhealthydad.com is live.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>From Oct 28 (reveal). Lines 1-3 are search terms. Line 4 is the trust signal: the misinformation-backlash trend, and 'AI Dad' shouldn't read as an AI persona. Category: Digital creator. Add the link once aidadhealthydad.com is live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Pinned / Highlights</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>From Nov 4: pin Scripts B, A, C on TikTok. Instagram Highlights: 'Start Here', '5AM Gym', 'AI Prompts', 'Diagnosis Log'.</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Pin Script B on TikTok now; add A and C after the reveal. Instagram Highlights: 'Start Here', '5AM Gym', 'AI Prompts', 'Diagnosis Log'.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2615,7 +2450,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>From Mon Nov 9 (after the teaser phase and reveal week; see Launch Phases). Weekly rhythm: Mon AI External Brain · Tue AI for Your Family · Wed 5AM Brain · Thu ADHD Dad in the Wild · Fri Late-Diagnosis Log · Sat NotebookLM + reply-to-comment video · Sun batch-film (the weekly ideas doc lands at 5 AM ET). 6 pillars × 15 starter ideas; fresh researched ideas arrive every Sunday. Ideas are story shapes: you supply the real story live.</t>
+          <t>From Mon Nov 2 (after the teaser phase and reveal week; see Launch Phases). Weekly rhythm: Mon AI External Brain · Tue AI for Your Family · Wed 5AM Brain · Thu ADHD Dad in the Wild · Fri Late-Diagnosis Log · Sat NotebookLM + reply-to-comment video · Sun batch-film (the weekly ideas doc lands at 5 AM ET). 6 pillars × 15 starter ideas; fresh researched ideas arrive every Sunday. Ideas are story shapes: you supply the real story live.</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2545,7 @@
 3) The school flyer trick: photo of the flyer, AI turns it into reminders. Save: the 3-step workflow.
 4) The worry sort: voice-memo everything on my mind, and AI sorts it into today / this week / not mine. Save: the sorting prompt.
 5) I asked AI if my channel name was trademarked: what it found, and what it said I still had to check myself. Save: the 'verify it yourself' list.
-6) AI built me a spreadsheet with 974 rows. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
+6) AI built me a spreadsheet with 956 rows. Here's how I made it useful: 'just tell me this week's 3 things'. Save: the shrink-it prompt.
 7) The 'am I sliding?' check-in: one sentence to AI when the old pattern starts, and it asks me 3 questions back. Save: the 3 questions.
 8) 'Remind me later' → a real calendar event in 10 seconds, hands-free. Save: the dictation phrasing that works.
 9) What I will NOT use AI for: talking to my kids, apologizing to my wife, health decisions. Save: my human-only list.
@@ -3582,12 +3417,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>The teaser plan assumes Scripts B, C and A haven't been posted yet (the old calendar had them on Oct 14-16).</t>
+          <t>Script B ('The Acronym') is already live on TikTok. It names ADHD and AI but no tools, so it fits the teaser rule.</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>If any are live, the reveal already happened on that account: either make them private before teaser 1, or skip Phase 1 and keep the normal rhythm.</t>
+          <t>If anything else already posted shows a tool or the workflow, the reveal has partly happened: keep the Oct 28 date anyway.</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3434,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Phase 1 length (2 weeks, 12 posts) is a judgment call. No study measures teaser length for new accounts; it rests on TikTok's description of how videos get matched, new-account guides (test phase of about 10-20 videos, traction about 90 days) and practitioner teaser advice (2-3 weeks). Those numbers come from search summaries, not pages I opened.</t>
+          <t>Phase 1 length (6 posts, Oct 21-27) is your decision. It sits inside what the research supports: no study measures teaser length; practitioner advice gives 2-3 weeks as the upper limit; a new account has no audience to keep waiting; and with ADHD and AI visible from post 1, the short phase costs nothing in discovery. Those numbers come from search summaries, not pages I opened.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -7370,7 +7205,7 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
@@ -7378,7 +7213,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Phase 1 teases real-life moments and results without explaining the mechanism. Phase 2 reveals it: the AI-and-ADHD angle. The phase length below was chosen from research on new accounts (sources in the Sources section, marked 'Launch phases'). No study measures teaser length directly, so the call is reasoned from what is known.</t>
+          <t>Phase 1 teases real results without showing how they happen. Phase 2 reveals the setup: the specific AI tools and the workflow. The same rule applies on TikTok and Instagram.</t>
         </is>
       </c>
     </row>
@@ -7402,34 +7237,34 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Phase 1: teaser length</t>
+          <t>What's open, what's hidden</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2 weeks, 12 posts: Wed Oct 21 to Tue Nov 3, Monday to Saturday at 7:00 AM ET. Sundays are for filming.</t>
+          <t>Open from day one: ADHD, being late-diagnosed, and 'I use AI'. Hidden until Oct 28: the specific tools (app names, logos, screens) and the workflow (what you type, the steps).</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Short on purpose. A brand-new account has no audience to keep in suspense: most viewers see one video, not the series. TikTok matches videos to viewers using captions, sounds, hashtags and what people watch (TikTok newsroom), so every week without 'ADHD dad' in the words is a week the app can't tell who your videos are for. Practitioner guidance on teasers says 2-3 weeks before interest wears out; one curiosity-marketing piece says people check out after 2 weeks. I took the low end.</t>
+          <t>The ADHD-and-AI angle is the account's search identity, so it stays visible. The curiosity hook is 'which tools, and how?', and that's what the reveal pays off.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Why not shorter</t>
+          <t>Phase 1: teaser length</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Not 1 week (6 posts).</t>
+          <t>6 posts: Wed Oct 21, Thu 22, Fri 23, Sat 24, Mon 26, Tue 27, at 7:00 AM ET. Sunday Oct 25 is for filming.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>New-account guides describe roughly the first 10-20 videos as the test phase where the app is still working out who to show you to (a creator rule of thumb, not TikTok data). 12 teasers sit inside that window and give enough posts for a returning viewer to notice a pattern before the reveal lands on video 13.</t>
+          <t>Your call, and it fits the research. A brand-new account has no audience to hold in suspense: most viewers see one video, not the series. Practitioner teaser advice gives 2-3 weeks as the most a teaser should run, not a minimum. And because ADHD and AI are visible from post 1, TikTok can match you to the right viewers (it uses captions, sounds and hashtags) during the teasers too, so a short phase costs nothing in discovery.</t>
         </is>
       </c>
     </row>
@@ -7441,12 +7276,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>After at least 6 teasers, if 3 or more posts get comments asking how or why, reveal on the next posting day.</t>
+          <t>After at least 3 teasers, if 2 or more posts get comments asking which app or how, reveal on the next posting day.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Those comments are the curiosity the teaser phase exists to create. Once it shows up, cashing it in beats making people wait.</t>
+          <t>Those comments are exactly the curiosity the teasers are for. Cash it in.</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7298,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Low views in weeks 1-2 are normal for any new account: growth guides put meaningful traction at about 90 days of consistent posting. Keeping the mystery longer won't fix that, and it keeps your search words hidden.</t>
+          <t>Low views in the first weeks are normal for any new account: growth guides put real traction at about 90 days. Holding the reveal back won't change that.</t>
         </is>
       </c>
     </row>
@@ -7475,12 +7310,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Wed Nov 4 Script B ('The Acronym') · Thu Nov 5 Script A ('The Parking Lot') · Fri Nov 6 Script C ('5:40 AM') · Sat Nov 7 reply video to the best 'how?' comment from Phase 1.</t>
+          <t>Wed Oct 28: the reveal video, the actual tools and one real example of each, on screen. Thu Oct 29: Script A ('The Parking Lot'). Fri Oct 30: Script C ('5:40 AM'). Sat Oct 31: reply video to the best 'which app?' comment.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>The account name is already the clue (the initials spell ADHD), so B pays it off. Switch both bios to the reveal versions the morning of Nov 4. Pin B, A and C.</t>
+          <t>Script B is already live on TikTok and did the ADHD-and-AI intro, so the reveal is about the setup. Switch both bios to the reveal versions the morning of Oct 28. Pin B, A and C.</t>
         </is>
       </c>
     </row>
@@ -7492,12 +7327,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>From Mon Nov 9: the 6-pillar weekly rhythm in Content Pillars.</t>
+          <t>From Mon Nov 2: the 6-pillar weekly rhythm in Content Pillars.</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Each teaser maps to a pillar, so every Phase 1 moment gets a full 'here's how' video later.</t>
+          <t>Each teaser maps to a pillar, so every teaser moment later gets its full 'here's how' video.</t>
         </is>
       </c>
     </row>
@@ -7509,12 +7344,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Show a real moment and a real result. Say what changed, never why. No 'ADHD', 'AI', 'diagnosis' or app names in the video, captions, on-screen text or hashtags. End each teaser with a line like 'More on that soon.'</t>
+          <t>Show a real moment and a real result. Saying ADHD or 'AI did this' is fine. Never name or show the tool, the screen, or the steps. End each teaser with a line like 'I'll show you exactly how on Oct 28.'</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>The mystery has to come from the result, not from withholding the point: each video still has to be worth watching on its own.</t>
+          <t>Each video still has to be worth watching on its own.</t>
         </is>
       </c>
     </row>
@@ -7526,7 +7361,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Only real results, no invented timelines. If someone asks how, reply: 'Telling the whole story on Nov 4.' Never deny it or make up a different reason.</t>
+          <t>Only real results, no invented timelines. If someone asks which app, reply: 'Showing the whole setup on Oct 28.' Never make up a different answer.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -7560,12 +7395,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Results and dad tags only, e.g. #dadsoftiktok #dadlife #5amclub #morningroutine. Re-check them weekly.</t>
+          <t>ADHD, dad and results tags are fine, e.g. #adhddad #adultadhd #dadsoftiktok #5amclub. No tool or app tags until Oct 28. Re-check them weekly.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Keeps the mechanism hidden while still giving the app words to match you on.</t>
+          <t>Keeps the setup hidden while the account's search words stay visible.</t>
         </is>
       </c>
     </row>

</xml_diff>